<commit_message>
Fix NR alteration fenestration U-factor checks for added vs altered (#1074).
Apply 0.47 only to newly added vertical fenestration and 0.58 to altered area over 150 sf, instead of blending New+Altered against 0.47. Also recognize .cibd25x in the test harness IBD regex.
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330A60BE-61FF-4FCF-8636-1F7798A2CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FEEA15-8B92-4F66-9DC4-44DB8FFB9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5910" yWindow="1080" windowWidth="17145" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1170" windowWidth="20535" windowHeight="14760" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8118" uniqueCount="1184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8116" uniqueCount="1183">
   <si>
     <t>;</t>
   </si>
@@ -3805,9 +3805,6 @@
   </si>
   <si>
     <t>SegIdx</t>
-  </si>
-  <si>
-    <t>08/26/26 - SAC - updated T24RDHW_LoopPipeSize table 2025+ Branch pipe diam from 1.5 (old value) to 0.75 for consistency w/ ACM AppB (dev #943)</t>
   </si>
 </sst>
 </file>
@@ -4491,7 +4488,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5028,6 +5025,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75206,7 +75206,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.85546875" customWidth="1"/>
@@ -75258,7 +75258,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75266,60 +75266,63 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="D7" t="s">
-        <v>1174</v>
-      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>494</v>
-      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
-      <c r="B13" t="s">
-        <v>6</v>
+      <c r="C13">
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -75327,10 +75330,10 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>496</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -75338,10 +75341,10 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>1180</v>
+        <v>497</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -75349,22 +75352,16 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>497</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17" t="s">
-        <v>1181</v>
-      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -75375,92 +75372,105 @@
       <c r="A19" t="s">
         <v>0</v>
       </c>
+      <c r="B19" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" t="s">
-        <v>500</v>
-      </c>
+      <c r="B20" s="145" t="s">
+        <v>544</v>
+      </c>
+      <c r="C20" s="145"/>
+      <c r="D20" s="146"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="145" t="s">
-        <v>544</v>
-      </c>
-      <c r="C21" s="145"/>
-      <c r="D21" s="146"/>
-      <c r="E21" s="146"/>
-      <c r="F21" s="146"/>
+      <c r="C21" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D21" s="147" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E21" s="147" t="s">
+        <v>498</v>
+      </c>
+      <c r="F21" s="147" t="s">
+        <v>1182</v>
+      </c>
+      <c r="G21" s="147" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D22" s="147" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E22" s="147" t="s">
-        <v>498</v>
-      </c>
-      <c r="F22" s="147" t="s">
-        <v>1182</v>
-      </c>
-      <c r="G22" s="147" t="s">
-        <v>499</v>
+      <c r="C22" s="1" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="F22" s="28">
+        <v>0</v>
+      </c>
+      <c r="G22" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="1" t="s">
-        <v>1175</v>
+      <c r="C23" s="6" t="str">
+        <f>C22</f>
+        <v>&lt;2024</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="28">
-        <v>0</v>
-      </c>
-      <c r="G23" s="28">
-        <v>1.5</v>
+      <c r="F23" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="6" t="str">
-        <f>C23</f>
+        <f t="shared" ref="C24:C30" si="0">C23</f>
         <v>&lt;2024</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G24" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C25" s="6" t="str">
-        <f t="shared" ref="C25:C31" si="0">C24</f>
+        <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G25" s="1">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -75472,13 +75482,13 @@
         <v>353</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G26" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -75490,13 +75500,13 @@
         <v>353</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G27" s="1">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -75508,13 +75518,13 @@
         <v>353</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G28" s="1">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -75526,66 +75536,65 @@
         <v>353</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G29" s="1">
-        <v>3.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="6" t="str">
+      <c r="C30" s="36" t="str">
         <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="E30" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="G30" s="1">
-        <v>4</v>
+      <c r="G30" s="4">
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31" s="36" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;2024</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E31" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="F31" s="4" t="s">
+      <c r="D31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G31" s="4">
-        <v>5</v>
+      <c r="E31" s="28" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F31" s="28">
+        <v>0</v>
+      </c>
+      <c r="G31" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E32" s="28" t="s">
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="F32" s="28">
-        <v>0</v>
-      </c>
-      <c r="G32" s="28">
-        <v>0.75</v>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="G32" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
@@ -75599,10 +75608,10 @@
         <v>1178</v>
       </c>
       <c r="F33" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.25">
@@ -75612,13 +75621,13 @@
       <c r="D34" s="1">
         <v>0</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F34" s="1">
-        <v>2</v>
-      </c>
-      <c r="G34" s="1">
+      <c r="F34" s="22">
+        <v>3</v>
+      </c>
+      <c r="G34" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -75629,14 +75638,14 @@
       <c r="D35" s="1">
         <v>0</v>
       </c>
-      <c r="E35" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F35" s="22">
-        <v>3</v>
-      </c>
-      <c r="G35" s="22">
-        <v>0.75</v>
+      <c r="E35" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
@@ -75650,10 +75659,10 @@
         <v>502</v>
       </c>
       <c r="F36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.25">
@@ -75663,14 +75672,14 @@
       <c r="D37" s="1">
         <v>0</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F37" s="1">
-        <v>2</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
+      <c r="F37" s="22">
+        <v>3</v>
+      </c>
+      <c r="G37" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
@@ -75680,14 +75689,14 @@
       <c r="D38" s="1">
         <v>0</v>
       </c>
-      <c r="E38" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F38" s="22">
-        <v>3</v>
-      </c>
-      <c r="G38" s="22">
-        <v>0.75</v>
+      <c r="E38" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
@@ -75701,10 +75710,10 @@
         <v>503</v>
       </c>
       <c r="F39" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
@@ -75714,13 +75723,13 @@
       <c r="D40" s="1">
         <v>0</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F40" s="1">
-        <v>2</v>
-      </c>
-      <c r="G40" s="1">
+      <c r="F40" s="22">
+        <v>3</v>
+      </c>
+      <c r="G40" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75731,14 +75740,14 @@
       <c r="D41" s="1">
         <v>0</v>
       </c>
-      <c r="E41" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F41" s="22">
-        <v>3</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.5</v>
+      <c r="E41" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1">
+        <v>2.5</v>
       </c>
     </row>
     <row r="42" spans="3:7" x14ac:dyDescent="0.25">
@@ -75752,10 +75761,10 @@
         <v>1179</v>
       </c>
       <c r="F42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="1">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.25">
@@ -75765,13 +75774,13 @@
       <c r="D43" s="1">
         <v>0</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F43" s="1">
-        <v>2</v>
-      </c>
-      <c r="G43" s="1">
+      <c r="F43" s="22">
+        <v>3</v>
+      </c>
+      <c r="G43" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75782,14 +75791,14 @@
       <c r="D44" s="1">
         <v>0</v>
       </c>
-      <c r="E44" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F44" s="22">
+      <c r="E44" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F44" s="1">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1">
         <v>3</v>
-      </c>
-      <c r="G44" s="22">
-        <v>1.5</v>
       </c>
     </row>
     <row r="45" spans="3:7" x14ac:dyDescent="0.25">
@@ -75803,10 +75812,10 @@
         <v>505</v>
       </c>
       <c r="F45" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="46" spans="3:7" x14ac:dyDescent="0.25">
@@ -75816,13 +75825,13 @@
       <c r="D46" s="1">
         <v>0</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F46" s="1">
-        <v>2</v>
-      </c>
-      <c r="G46" s="1">
+      <c r="F46" s="22">
+        <v>3</v>
+      </c>
+      <c r="G46" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75833,14 +75842,14 @@
       <c r="D47" s="1">
         <v>0</v>
       </c>
-      <c r="E47" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F47" s="22">
-        <v>3</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.5</v>
+      <c r="E47" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1">
+        <v>3.5</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.25">
@@ -75854,10 +75863,10 @@
         <v>506</v>
       </c>
       <c r="F48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="1">
-        <v>3.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="3:7" x14ac:dyDescent="0.25">
@@ -75867,14 +75876,14 @@
       <c r="D49" s="1">
         <v>0</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F49" s="1">
-        <v>2</v>
-      </c>
-      <c r="G49" s="1">
-        <v>2</v>
+      <c r="F49" s="22">
+        <v>3</v>
+      </c>
+      <c r="G49" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="50" spans="3:7" x14ac:dyDescent="0.25">
@@ -75884,14 +75893,14 @@
       <c r="D50" s="1">
         <v>0</v>
       </c>
-      <c r="E50" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F50" s="22">
-        <v>3</v>
-      </c>
-      <c r="G50" s="22">
-        <v>1.5</v>
+      <c r="E50" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+      <c r="G50" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="3:7" x14ac:dyDescent="0.25">
@@ -75905,10 +75914,10 @@
         <v>507</v>
       </c>
       <c r="F51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="3:7" x14ac:dyDescent="0.25">
@@ -75918,14 +75927,14 @@
       <c r="D52" s="1">
         <v>0</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F52" s="1">
-        <v>2</v>
-      </c>
-      <c r="G52" s="1">
-        <v>2</v>
+      <c r="F52" s="22">
+        <v>3</v>
+      </c>
+      <c r="G52" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="53" spans="3:7" x14ac:dyDescent="0.25">
@@ -75935,14 +75944,14 @@
       <c r="D53" s="1">
         <v>0</v>
       </c>
-      <c r="E53" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F53" s="22">
-        <v>3</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.5</v>
+      <c r="E53" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F53" s="1">
+        <v>1</v>
+      </c>
+      <c r="G53" s="1">
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="3:7" x14ac:dyDescent="0.25">
@@ -75956,10 +75965,10 @@
         <v>508</v>
       </c>
       <c r="F54" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="3:7" x14ac:dyDescent="0.25">
@@ -75969,82 +75978,82 @@
       <c r="D55" s="1">
         <v>0</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55" s="22">
+        <v>3</v>
+      </c>
+      <c r="G55" s="22">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D56" s="234">
+        <v>0</v>
+      </c>
+      <c r="E56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F56" s="234">
+        <v>1</v>
+      </c>
+      <c r="G56" s="234">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D57" s="234">
+        <v>0</v>
+      </c>
+      <c r="E57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F57" s="234">
         <v>2</v>
       </c>
-      <c r="G55" s="1">
+      <c r="G57" s="234">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D56" s="1">
-        <v>0</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F56" s="22">
+      <c r="D58" s="22">
+        <v>0</v>
+      </c>
+      <c r="E58" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="F58" s="22">
         <v>3</v>
       </c>
-      <c r="G56" s="22">
+      <c r="G58" s="22">
         <v>1.5</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D57" s="1">
-        <v>0</v>
-      </c>
-      <c r="E57" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F57" s="1">
-        <v>1</v>
-      </c>
-      <c r="G57" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="1">
-        <v>0</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F58" s="1">
-        <v>2</v>
-      </c>
-      <c r="G58" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="22">
-        <v>0</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="F59" s="22">
-        <v>3</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.5</v>
+      <c r="E59" s="1" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F59" s="1">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="3:7" x14ac:dyDescent="0.25">
@@ -76058,10 +76067,10 @@
         <v>1178</v>
       </c>
       <c r="F60" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="61" spans="3:7" x14ac:dyDescent="0.25">
@@ -76071,13 +76080,13 @@
       <c r="D61" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F61" s="1">
-        <v>2</v>
-      </c>
-      <c r="G61" s="1">
+      <c r="F61" s="22">
+        <v>3</v>
+      </c>
+      <c r="G61" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -76088,14 +76097,14 @@
       <c r="D62" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E62" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F62" s="22">
-        <v>3</v>
-      </c>
-      <c r="G62" s="22">
-        <v>0.75</v>
+      <c r="E62" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F62" s="1">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="63" spans="3:7" x14ac:dyDescent="0.25">
@@ -76109,10 +76118,10 @@
         <v>502</v>
       </c>
       <c r="F63" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="3:7" x14ac:dyDescent="0.25">
@@ -76122,14 +76131,14 @@
       <c r="D64" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F64" s="1">
-        <v>2</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
+      <c r="F64" s="22">
+        <v>3</v>
+      </c>
+      <c r="G64" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="65" spans="3:7" x14ac:dyDescent="0.25">
@@ -76139,14 +76148,14 @@
       <c r="D65" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E65" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F65" s="22">
-        <v>3</v>
-      </c>
-      <c r="G65" s="22">
-        <v>0.75</v>
+      <c r="E65" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F65" s="1">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="66" spans="3:7" x14ac:dyDescent="0.25">
@@ -76160,7 +76169,7 @@
         <v>503</v>
       </c>
       <c r="F66" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="1">
         <v>1.5</v>
@@ -76173,14 +76182,14 @@
       <c r="D67" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E67" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F67" s="1">
-        <v>2</v>
-      </c>
-      <c r="G67" s="1">
-        <v>1.5</v>
+      <c r="F67" s="22">
+        <v>3</v>
+      </c>
+      <c r="G67" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -76190,14 +76199,14 @@
       <c r="D68" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E68" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F68" s="22">
-        <v>3</v>
-      </c>
-      <c r="G68" s="22">
-        <v>1</v>
+      <c r="E68" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F68" s="1">
+        <v>1</v>
+      </c>
+      <c r="G68" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="69" spans="3:7" x14ac:dyDescent="0.25">
@@ -76211,7 +76220,7 @@
         <v>1179</v>
       </c>
       <c r="F69" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G69" s="1">
         <v>1.5</v>
@@ -76224,14 +76233,14 @@
       <c r="D70" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E70" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F70" s="1">
-        <v>2</v>
-      </c>
-      <c r="G70" s="1">
-        <v>1.5</v>
+      <c r="F70" s="22">
+        <v>3</v>
+      </c>
+      <c r="G70" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="3:7" x14ac:dyDescent="0.25">
@@ -76241,14 +76250,14 @@
       <c r="D71" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E71" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F71" s="22">
-        <v>3</v>
-      </c>
-      <c r="G71" s="22">
-        <v>1</v>
+      <c r="E71" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F71" s="1">
+        <v>1</v>
+      </c>
+      <c r="G71" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="3:7" x14ac:dyDescent="0.25">
@@ -76262,10 +76271,10 @@
         <v>505</v>
       </c>
       <c r="F72" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="73" spans="3:7" x14ac:dyDescent="0.25">
@@ -76275,14 +76284,14 @@
       <c r="D73" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E73" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F73" s="1">
-        <v>2</v>
-      </c>
-      <c r="G73" s="1">
-        <v>1.5</v>
+      <c r="F73" s="22">
+        <v>3</v>
+      </c>
+      <c r="G73" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="3:7" x14ac:dyDescent="0.25">
@@ -76292,14 +76301,14 @@
       <c r="D74" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E74" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F74" s="22">
+      <c r="E74" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F74" s="1">
+        <v>1</v>
+      </c>
+      <c r="G74" s="1">
         <v>3</v>
-      </c>
-      <c r="G74" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="75" spans="3:7" x14ac:dyDescent="0.25">
@@ -76313,10 +76322,10 @@
         <v>506</v>
       </c>
       <c r="F75" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="76" spans="3:7" x14ac:dyDescent="0.25">
@@ -76326,14 +76335,14 @@
       <c r="D76" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="E76" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F76" s="1">
-        <v>2</v>
-      </c>
-      <c r="G76" s="1">
-        <v>1.5</v>
+      <c r="F76" s="22">
+        <v>3</v>
+      </c>
+      <c r="G76" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="3:7" x14ac:dyDescent="0.25">
@@ -76343,14 +76352,14 @@
       <c r="D77" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E77" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F77" s="22">
+      <c r="E77" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F77" s="1">
+        <v>1</v>
+      </c>
+      <c r="G77" s="1">
         <v>3</v>
-      </c>
-      <c r="G77" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="78" spans="3:7" x14ac:dyDescent="0.25">
@@ -76364,10 +76373,10 @@
         <v>507</v>
       </c>
       <c r="F78" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="79" spans="3:7" x14ac:dyDescent="0.25">
@@ -76377,14 +76386,14 @@
       <c r="D79" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E79" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F79" s="1">
-        <v>2</v>
-      </c>
-      <c r="G79" s="1">
-        <v>1.5</v>
+      <c r="F79" s="22">
+        <v>3</v>
+      </c>
+      <c r="G79" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="3:7" x14ac:dyDescent="0.25">
@@ -76394,14 +76403,14 @@
       <c r="D80" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E80" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F80" s="22">
+      <c r="E80" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F80" s="1">
+        <v>1</v>
+      </c>
+      <c r="G80" s="1">
         <v>3</v>
-      </c>
-      <c r="G80" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -76415,10 +76424,10 @@
         <v>508</v>
       </c>
       <c r="F81" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G81" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -76428,104 +76437,92 @@
       <c r="D82" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E82" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F82" s="1">
+      <c r="F82" s="22">
+        <v>3</v>
+      </c>
+      <c r="G82" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F83" s="234">
+        <v>1</v>
+      </c>
+      <c r="G83" s="234">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F84" s="234">
         <v>2</v>
       </c>
-      <c r="G82" s="1">
+      <c r="G84" s="234">
         <v>1.5</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C83" s="1" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E83" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F83" s="22">
+      <c r="E85" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="F85" s="4">
         <v>3</v>
       </c>
-      <c r="G83" s="22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C84" s="1" t="s">
+      <c r="G85" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="E86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F84" s="1">
-        <v>1</v>
-      </c>
-      <c r="G84" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C85" s="1" t="s">
+      <c r="F86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F85" s="1">
-        <v>2</v>
-      </c>
-      <c r="G85" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="D86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="E86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="F86" s="4">
-        <v>3</v>
-      </c>
-      <c r="G86" s="4">
-        <v>1</v>
+      <c r="G86" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G87" s="1">
-        <v>6</v>
+      <c r="B87" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
-        <v>50</v>
+      <c r="A88" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -76537,53 +76534,66 @@
       <c r="A90" t="s">
         <v>0</v>
       </c>
+      <c r="B90" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>0</v>
-      </c>
-      <c r="B91" t="s">
-        <v>1159</v>
-      </c>
+      <c r="B91" s="145" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C91" s="145"/>
+      <c r="D91" s="146"/>
+      <c r="E91" s="146"/>
+      <c r="F91" s="146"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B92" s="145" t="s">
-        <v>1160</v>
-      </c>
-      <c r="C92" s="145"/>
-      <c r="D92" s="146"/>
-      <c r="E92" s="146"/>
-      <c r="F92" s="146"/>
+      <c r="C92" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D92" s="229" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E92" s="147" t="s">
+        <v>1162</v>
+      </c>
+      <c r="F92" s="229" t="s">
+        <v>1166</v>
+      </c>
+      <c r="G92" s="148" t="s">
+        <v>1168</v>
+      </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C93" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D93" s="229" t="s">
-        <v>1161</v>
-      </c>
-      <c r="E93" s="147" t="s">
-        <v>1162</v>
-      </c>
-      <c r="F93" s="229" t="s">
-        <v>1166</v>
-      </c>
-      <c r="G93" s="148" t="s">
-        <v>1168</v>
+      <c r="C93" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D93" s="230" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F93" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G93" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C94" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D94" s="230" t="s">
-        <v>1164</v>
-      </c>
-      <c r="E94" s="1" t="s">
+      <c r="D94" s="232" t="str">
+        <f>D93</f>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F94" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G94" s="1">
         <v>1</v>
@@ -76594,17 +76604,17 @@
         <v>353</v>
       </c>
       <c r="D95" s="232" t="str">
-        <f>D94</f>
+        <f t="shared" ref="D95:D98" si="1">D94</f>
         <v>MPassInteg</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F95" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G95" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -76612,17 +76622,17 @@
         <v>353</v>
       </c>
       <c r="D96" s="232" t="str">
-        <f t="shared" ref="D96:D99" si="1">D95</f>
+        <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E96" s="6" t="s">
-        <v>1163</v>
+      <c r="E96" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F96" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G96" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="3:7" x14ac:dyDescent="0.25">
@@ -76633,67 +76643,67 @@
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E97" s="1" t="s">
+      <c r="E97" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F97" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G97" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C98" s="1" t="s">
+      <c r="C98" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D98" s="232" t="str">
+      <c r="D98" s="233" t="str">
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E98" s="6" t="s">
+      <c r="E98" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F98" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G98" s="1">
-        <v>1</v>
+      <c r="F98" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G98" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="99" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C99" s="22" t="s">
+      <c r="C99" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D99" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E99" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F99" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G99" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D99" s="230" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F99" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G99" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C100" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D100" s="230" t="s">
-        <v>1170</v>
-      </c>
-      <c r="E100" s="1" t="s">
+      <c r="D100" s="232" t="str">
+        <f>D99</f>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E100" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F100" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G100" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.25">
@@ -76701,17 +76711,17 @@
         <v>353</v>
       </c>
       <c r="D101" s="232" t="str">
-        <f>D100</f>
+        <f t="shared" ref="D101:D104" si="2">D100</f>
         <v>SPassPrim-PrimTank</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F101" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G101" s="1">
-        <v>1</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="102" spans="3:7" x14ac:dyDescent="0.25">
@@ -76719,17 +76729,17 @@
         <v>353</v>
       </c>
       <c r="D102" s="232" t="str">
-        <f t="shared" ref="D102:D105" si="2">D101</f>
+        <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E102" s="6" t="s">
-        <v>1163</v>
+      <c r="E102" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F102" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G102" s="1">
-        <v>1.1399999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="3:7" x14ac:dyDescent="0.25">
@@ -76740,67 +76750,67 @@
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E103" s="1" t="s">
+      <c r="E103" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F103" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G103" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C104" s="1" t="s">
+      <c r="C104" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D104" s="232" t="str">
+      <c r="D104" s="233" t="str">
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="E104" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F104" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G104" s="1">
-        <v>1</v>
+      <c r="F104" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G104" s="22">
+        <v>1.0900000000000001</v>
       </c>
     </row>
     <row r="105" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C105" s="22" t="s">
+      <c r="C105" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D105" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E105" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F105" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G105" s="22">
-        <v>1.0900000000000001</v>
+      <c r="D105" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F105" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G105" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C106" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D106" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="E106" s="1" t="s">
+      <c r="D106" s="232" t="str">
+        <f>D105</f>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E106" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F106" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G106" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.25">
@@ -76808,17 +76818,17 @@
         <v>353</v>
       </c>
       <c r="D107" s="232" t="str">
-        <f>D106</f>
+        <f t="shared" ref="D107:D110" si="3">D106</f>
         <v>MPassPrim-PrimTank</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F107" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G107" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.25">
@@ -76826,17 +76836,17 @@
         <v>353</v>
       </c>
       <c r="D108" s="232" t="str">
-        <f t="shared" ref="D108:D111" si="3">D107</f>
+        <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E108" s="6" t="s">
-        <v>1163</v>
+      <c r="E108" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F108" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G108" s="1">
-        <v>1.1499999999999999</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.25">
@@ -76847,67 +76857,67 @@
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="E109" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F109" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G109" s="1">
-        <v>0.98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C110" s="1" t="s">
+      <c r="C110" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D110" s="232" t="str">
+      <c r="D110" s="233" t="str">
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E110" s="6" t="s">
+      <c r="E110" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F110" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G110" s="1">
-        <v>1</v>
+      <c r="F110" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G110" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C111" s="22" t="s">
+      <c r="C111" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D111" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E111" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F111" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G111" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D111" s="230" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F111" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G111" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C112" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D112" s="230" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E112" s="1" t="s">
+      <c r="D112" s="232" t="str">
+        <f>D111</f>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E112" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F112" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G112" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -76915,17 +76925,17 @@
         <v>353</v>
       </c>
       <c r="D113" s="232" t="str">
-        <f>D112</f>
+        <f t="shared" ref="D113:D116" si="4">D112</f>
         <v>SPassPrim-SResist</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F113" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G113" s="1">
-        <v>1</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -76933,17 +76943,17 @@
         <v>353</v>
       </c>
       <c r="D114" s="232" t="str">
-        <f t="shared" ref="D114:D117" si="4">D113</f>
+        <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E114" s="6" t="s">
-        <v>1163</v>
+      <c r="E114" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F114" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G114" s="1">
-        <v>1.08</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -76954,67 +76964,67 @@
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E115" s="1" t="s">
+      <c r="E115" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F115" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G115" s="1">
-        <v>0.99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C116" s="1" t="s">
+      <c r="C116" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D116" s="232" t="str">
+      <c r="D116" s="233" t="str">
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E116" s="6" t="s">
+      <c r="E116" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F116" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G116" s="1">
-        <v>1</v>
+      <c r="F116" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G116" s="22">
+        <v>1.05</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C117" s="22" t="s">
+      <c r="C117" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D117" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E117" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F117" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G117" s="22">
-        <v>1.05</v>
+      <c r="D117" s="230" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F117" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G117" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D118" s="230" t="s">
-        <v>1173</v>
-      </c>
-      <c r="E118" s="1" t="s">
+      <c r="D118" s="232" t="str">
+        <f>D117</f>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F118" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G118" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -77022,17 +77032,17 @@
         <v>353</v>
       </c>
       <c r="D119" s="232" t="str">
-        <f>D118</f>
+        <f t="shared" ref="D119:D122" si="5">D118</f>
         <v>SPassPrim-Parallel</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F119" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G119" s="1">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -77040,17 +77050,17 @@
         <v>353</v>
       </c>
       <c r="D120" s="232" t="str">
-        <f t="shared" ref="D120:D123" si="5">D119</f>
+        <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E120" s="6" t="s">
-        <v>1163</v>
+      <c r="E120" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F120" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G120" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -77061,76 +77071,58 @@
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E121" s="1" t="s">
+      <c r="E121" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F121" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G121" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C122" s="1" t="s">
+      <c r="C122" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D122" s="232" t="str">
+      <c r="D122" s="233" t="str">
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E122" s="6" t="s">
+      <c r="E122" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F122" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G122" s="1">
-        <v>1</v>
+      <c r="F122" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G122" s="22">
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C123" s="22" t="s">
+      <c r="C123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D123" s="233" t="str">
-        <f t="shared" si="5"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E123" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F123" s="231" t="s">
+      <c r="D123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G123" s="22">
-        <v>1.1000000000000001</v>
+      <c r="E123" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F123" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G123" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F124" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G124" s="1">
-        <v>1</v>
+      <c r="B124" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="A125" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2025-CBECC-Schema Issue 64: - Modify XML output of multi-orientation Attributes from all uppercase (e.g., NORTH) to case sensitive with schema (e.g., North)
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330A60BE-61FF-4FCF-8636-1F7798A2CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FEEA15-8B92-4F66-9DC4-44DB8FFB9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5910" yWindow="1080" windowWidth="17145" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1170" windowWidth="20535" windowHeight="14760" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8118" uniqueCount="1184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8116" uniqueCount="1183">
   <si>
     <t>;</t>
   </si>
@@ -3805,9 +3805,6 @@
   </si>
   <si>
     <t>SegIdx</t>
-  </si>
-  <si>
-    <t>08/26/26 - SAC - updated T24RDHW_LoopPipeSize table 2025+ Branch pipe diam from 1.5 (old value) to 0.75 for consistency w/ ACM AppB (dev #943)</t>
   </si>
 </sst>
 </file>
@@ -4491,7 +4488,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5028,6 +5025,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75206,7 +75206,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.85546875" customWidth="1"/>
@@ -75258,7 +75258,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75266,60 +75266,63 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="D7" t="s">
-        <v>1174</v>
-      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>494</v>
-      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
-      <c r="B13" t="s">
-        <v>6</v>
+      <c r="C13">
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -75327,10 +75330,10 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>496</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -75338,10 +75341,10 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>1180</v>
+        <v>497</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -75349,22 +75352,16 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>497</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17" t="s">
-        <v>1181</v>
-      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -75375,92 +75372,105 @@
       <c r="A19" t="s">
         <v>0</v>
       </c>
+      <c r="B19" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" t="s">
-        <v>500</v>
-      </c>
+      <c r="B20" s="145" t="s">
+        <v>544</v>
+      </c>
+      <c r="C20" s="145"/>
+      <c r="D20" s="146"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="145" t="s">
-        <v>544</v>
-      </c>
-      <c r="C21" s="145"/>
-      <c r="D21" s="146"/>
-      <c r="E21" s="146"/>
-      <c r="F21" s="146"/>
+      <c r="C21" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D21" s="147" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E21" s="147" t="s">
+        <v>498</v>
+      </c>
+      <c r="F21" s="147" t="s">
+        <v>1182</v>
+      </c>
+      <c r="G21" s="147" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D22" s="147" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E22" s="147" t="s">
-        <v>498</v>
-      </c>
-      <c r="F22" s="147" t="s">
-        <v>1182</v>
-      </c>
-      <c r="G22" s="147" t="s">
-        <v>499</v>
+      <c r="C22" s="1" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="F22" s="28">
+        <v>0</v>
+      </c>
+      <c r="G22" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="1" t="s">
-        <v>1175</v>
+      <c r="C23" s="6" t="str">
+        <f>C22</f>
+        <v>&lt;2024</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="28">
-        <v>0</v>
-      </c>
-      <c r="G23" s="28">
-        <v>1.5</v>
+      <c r="F23" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="6" t="str">
-        <f>C23</f>
+        <f t="shared" ref="C24:C30" si="0">C23</f>
         <v>&lt;2024</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G24" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C25" s="6" t="str">
-        <f t="shared" ref="C25:C31" si="0">C24</f>
+        <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G25" s="1">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -75472,13 +75482,13 @@
         <v>353</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G26" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -75490,13 +75500,13 @@
         <v>353</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G27" s="1">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -75508,13 +75518,13 @@
         <v>353</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G28" s="1">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -75526,66 +75536,65 @@
         <v>353</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G29" s="1">
-        <v>3.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="6" t="str">
+      <c r="C30" s="36" t="str">
         <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="E30" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="G30" s="1">
-        <v>4</v>
+      <c r="G30" s="4">
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31" s="36" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;2024</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E31" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="F31" s="4" t="s">
+      <c r="D31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G31" s="4">
-        <v>5</v>
+      <c r="E31" s="28" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F31" s="28">
+        <v>0</v>
+      </c>
+      <c r="G31" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E32" s="28" t="s">
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="F32" s="28">
-        <v>0</v>
-      </c>
-      <c r="G32" s="28">
-        <v>0.75</v>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="G32" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
@@ -75599,10 +75608,10 @@
         <v>1178</v>
       </c>
       <c r="F33" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.25">
@@ -75612,13 +75621,13 @@
       <c r="D34" s="1">
         <v>0</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F34" s="1">
-        <v>2</v>
-      </c>
-      <c r="G34" s="1">
+      <c r="F34" s="22">
+        <v>3</v>
+      </c>
+      <c r="G34" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -75629,14 +75638,14 @@
       <c r="D35" s="1">
         <v>0</v>
       </c>
-      <c r="E35" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F35" s="22">
-        <v>3</v>
-      </c>
-      <c r="G35" s="22">
-        <v>0.75</v>
+      <c r="E35" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
@@ -75650,10 +75659,10 @@
         <v>502</v>
       </c>
       <c r="F36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.25">
@@ -75663,14 +75672,14 @@
       <c r="D37" s="1">
         <v>0</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F37" s="1">
-        <v>2</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
+      <c r="F37" s="22">
+        <v>3</v>
+      </c>
+      <c r="G37" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
@@ -75680,14 +75689,14 @@
       <c r="D38" s="1">
         <v>0</v>
       </c>
-      <c r="E38" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F38" s="22">
-        <v>3</v>
-      </c>
-      <c r="G38" s="22">
-        <v>0.75</v>
+      <c r="E38" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
@@ -75701,10 +75710,10 @@
         <v>503</v>
       </c>
       <c r="F39" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
@@ -75714,13 +75723,13 @@
       <c r="D40" s="1">
         <v>0</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F40" s="1">
-        <v>2</v>
-      </c>
-      <c r="G40" s="1">
+      <c r="F40" s="22">
+        <v>3</v>
+      </c>
+      <c r="G40" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75731,14 +75740,14 @@
       <c r="D41" s="1">
         <v>0</v>
       </c>
-      <c r="E41" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F41" s="22">
-        <v>3</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.5</v>
+      <c r="E41" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1">
+        <v>2.5</v>
       </c>
     </row>
     <row r="42" spans="3:7" x14ac:dyDescent="0.25">
@@ -75752,10 +75761,10 @@
         <v>1179</v>
       </c>
       <c r="F42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="1">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.25">
@@ -75765,13 +75774,13 @@
       <c r="D43" s="1">
         <v>0</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F43" s="1">
-        <v>2</v>
-      </c>
-      <c r="G43" s="1">
+      <c r="F43" s="22">
+        <v>3</v>
+      </c>
+      <c r="G43" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75782,14 +75791,14 @@
       <c r="D44" s="1">
         <v>0</v>
       </c>
-      <c r="E44" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F44" s="22">
+      <c r="E44" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F44" s="1">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1">
         <v>3</v>
-      </c>
-      <c r="G44" s="22">
-        <v>1.5</v>
       </c>
     </row>
     <row r="45" spans="3:7" x14ac:dyDescent="0.25">
@@ -75803,10 +75812,10 @@
         <v>505</v>
       </c>
       <c r="F45" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="46" spans="3:7" x14ac:dyDescent="0.25">
@@ -75816,13 +75825,13 @@
       <c r="D46" s="1">
         <v>0</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F46" s="1">
-        <v>2</v>
-      </c>
-      <c r="G46" s="1">
+      <c r="F46" s="22">
+        <v>3</v>
+      </c>
+      <c r="G46" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75833,14 +75842,14 @@
       <c r="D47" s="1">
         <v>0</v>
       </c>
-      <c r="E47" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F47" s="22">
-        <v>3</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.5</v>
+      <c r="E47" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1">
+        <v>3.5</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.25">
@@ -75854,10 +75863,10 @@
         <v>506</v>
       </c>
       <c r="F48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="1">
-        <v>3.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="3:7" x14ac:dyDescent="0.25">
@@ -75867,14 +75876,14 @@
       <c r="D49" s="1">
         <v>0</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F49" s="1">
-        <v>2</v>
-      </c>
-      <c r="G49" s="1">
-        <v>2</v>
+      <c r="F49" s="22">
+        <v>3</v>
+      </c>
+      <c r="G49" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="50" spans="3:7" x14ac:dyDescent="0.25">
@@ -75884,14 +75893,14 @@
       <c r="D50" s="1">
         <v>0</v>
       </c>
-      <c r="E50" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F50" s="22">
-        <v>3</v>
-      </c>
-      <c r="G50" s="22">
-        <v>1.5</v>
+      <c r="E50" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+      <c r="G50" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="3:7" x14ac:dyDescent="0.25">
@@ -75905,10 +75914,10 @@
         <v>507</v>
       </c>
       <c r="F51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="3:7" x14ac:dyDescent="0.25">
@@ -75918,14 +75927,14 @@
       <c r="D52" s="1">
         <v>0</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F52" s="1">
-        <v>2</v>
-      </c>
-      <c r="G52" s="1">
-        <v>2</v>
+      <c r="F52" s="22">
+        <v>3</v>
+      </c>
+      <c r="G52" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="53" spans="3:7" x14ac:dyDescent="0.25">
@@ -75935,14 +75944,14 @@
       <c r="D53" s="1">
         <v>0</v>
       </c>
-      <c r="E53" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F53" s="22">
-        <v>3</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.5</v>
+      <c r="E53" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F53" s="1">
+        <v>1</v>
+      </c>
+      <c r="G53" s="1">
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="3:7" x14ac:dyDescent="0.25">
@@ -75956,10 +75965,10 @@
         <v>508</v>
       </c>
       <c r="F54" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="3:7" x14ac:dyDescent="0.25">
@@ -75969,82 +75978,82 @@
       <c r="D55" s="1">
         <v>0</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55" s="22">
+        <v>3</v>
+      </c>
+      <c r="G55" s="22">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D56" s="234">
+        <v>0</v>
+      </c>
+      <c r="E56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F56" s="234">
+        <v>1</v>
+      </c>
+      <c r="G56" s="234">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D57" s="234">
+        <v>0</v>
+      </c>
+      <c r="E57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F57" s="234">
         <v>2</v>
       </c>
-      <c r="G55" s="1">
+      <c r="G57" s="234">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D56" s="1">
-        <v>0</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F56" s="22">
+      <c r="D58" s="22">
+        <v>0</v>
+      </c>
+      <c r="E58" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="F58" s="22">
         <v>3</v>
       </c>
-      <c r="G56" s="22">
+      <c r="G58" s="22">
         <v>1.5</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D57" s="1">
-        <v>0</v>
-      </c>
-      <c r="E57" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F57" s="1">
-        <v>1</v>
-      </c>
-      <c r="G57" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="1">
-        <v>0</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F58" s="1">
-        <v>2</v>
-      </c>
-      <c r="G58" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="22">
-        <v>0</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="F59" s="22">
-        <v>3</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.5</v>
+      <c r="E59" s="1" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F59" s="1">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="3:7" x14ac:dyDescent="0.25">
@@ -76058,10 +76067,10 @@
         <v>1178</v>
       </c>
       <c r="F60" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="61" spans="3:7" x14ac:dyDescent="0.25">
@@ -76071,13 +76080,13 @@
       <c r="D61" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F61" s="1">
-        <v>2</v>
-      </c>
-      <c r="G61" s="1">
+      <c r="F61" s="22">
+        <v>3</v>
+      </c>
+      <c r="G61" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -76088,14 +76097,14 @@
       <c r="D62" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E62" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F62" s="22">
-        <v>3</v>
-      </c>
-      <c r="G62" s="22">
-        <v>0.75</v>
+      <c r="E62" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F62" s="1">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="63" spans="3:7" x14ac:dyDescent="0.25">
@@ -76109,10 +76118,10 @@
         <v>502</v>
       </c>
       <c r="F63" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="3:7" x14ac:dyDescent="0.25">
@@ -76122,14 +76131,14 @@
       <c r="D64" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F64" s="1">
-        <v>2</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
+      <c r="F64" s="22">
+        <v>3</v>
+      </c>
+      <c r="G64" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="65" spans="3:7" x14ac:dyDescent="0.25">
@@ -76139,14 +76148,14 @@
       <c r="D65" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E65" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F65" s="22">
-        <v>3</v>
-      </c>
-      <c r="G65" s="22">
-        <v>0.75</v>
+      <c r="E65" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F65" s="1">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="66" spans="3:7" x14ac:dyDescent="0.25">
@@ -76160,7 +76169,7 @@
         <v>503</v>
       </c>
       <c r="F66" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="1">
         <v>1.5</v>
@@ -76173,14 +76182,14 @@
       <c r="D67" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E67" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F67" s="1">
-        <v>2</v>
-      </c>
-      <c r="G67" s="1">
-        <v>1.5</v>
+      <c r="F67" s="22">
+        <v>3</v>
+      </c>
+      <c r="G67" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -76190,14 +76199,14 @@
       <c r="D68" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E68" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F68" s="22">
-        <v>3</v>
-      </c>
-      <c r="G68" s="22">
-        <v>1</v>
+      <c r="E68" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F68" s="1">
+        <v>1</v>
+      </c>
+      <c r="G68" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="69" spans="3:7" x14ac:dyDescent="0.25">
@@ -76211,7 +76220,7 @@
         <v>1179</v>
       </c>
       <c r="F69" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G69" s="1">
         <v>1.5</v>
@@ -76224,14 +76233,14 @@
       <c r="D70" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E70" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F70" s="1">
-        <v>2</v>
-      </c>
-      <c r="G70" s="1">
-        <v>1.5</v>
+      <c r="F70" s="22">
+        <v>3</v>
+      </c>
+      <c r="G70" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="3:7" x14ac:dyDescent="0.25">
@@ -76241,14 +76250,14 @@
       <c r="D71" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E71" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F71" s="22">
-        <v>3</v>
-      </c>
-      <c r="G71" s="22">
-        <v>1</v>
+      <c r="E71" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F71" s="1">
+        <v>1</v>
+      </c>
+      <c r="G71" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="3:7" x14ac:dyDescent="0.25">
@@ -76262,10 +76271,10 @@
         <v>505</v>
       </c>
       <c r="F72" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="73" spans="3:7" x14ac:dyDescent="0.25">
@@ -76275,14 +76284,14 @@
       <c r="D73" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E73" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F73" s="1">
-        <v>2</v>
-      </c>
-      <c r="G73" s="1">
-        <v>1.5</v>
+      <c r="F73" s="22">
+        <v>3</v>
+      </c>
+      <c r="G73" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="3:7" x14ac:dyDescent="0.25">
@@ -76292,14 +76301,14 @@
       <c r="D74" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E74" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F74" s="22">
+      <c r="E74" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F74" s="1">
+        <v>1</v>
+      </c>
+      <c r="G74" s="1">
         <v>3</v>
-      </c>
-      <c r="G74" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="75" spans="3:7" x14ac:dyDescent="0.25">
@@ -76313,10 +76322,10 @@
         <v>506</v>
       </c>
       <c r="F75" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="76" spans="3:7" x14ac:dyDescent="0.25">
@@ -76326,14 +76335,14 @@
       <c r="D76" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="E76" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F76" s="1">
-        <v>2</v>
-      </c>
-      <c r="G76" s="1">
-        <v>1.5</v>
+      <c r="F76" s="22">
+        <v>3</v>
+      </c>
+      <c r="G76" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="3:7" x14ac:dyDescent="0.25">
@@ -76343,14 +76352,14 @@
       <c r="D77" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E77" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F77" s="22">
+      <c r="E77" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F77" s="1">
+        <v>1</v>
+      </c>
+      <c r="G77" s="1">
         <v>3</v>
-      </c>
-      <c r="G77" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="78" spans="3:7" x14ac:dyDescent="0.25">
@@ -76364,10 +76373,10 @@
         <v>507</v>
       </c>
       <c r="F78" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="79" spans="3:7" x14ac:dyDescent="0.25">
@@ -76377,14 +76386,14 @@
       <c r="D79" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E79" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F79" s="1">
-        <v>2</v>
-      </c>
-      <c r="G79" s="1">
-        <v>1.5</v>
+      <c r="F79" s="22">
+        <v>3</v>
+      </c>
+      <c r="G79" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="3:7" x14ac:dyDescent="0.25">
@@ -76394,14 +76403,14 @@
       <c r="D80" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E80" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F80" s="22">
+      <c r="E80" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F80" s="1">
+        <v>1</v>
+      </c>
+      <c r="G80" s="1">
         <v>3</v>
-      </c>
-      <c r="G80" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -76415,10 +76424,10 @@
         <v>508</v>
       </c>
       <c r="F81" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G81" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -76428,104 +76437,92 @@
       <c r="D82" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E82" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F82" s="1">
+      <c r="F82" s="22">
+        <v>3</v>
+      </c>
+      <c r="G82" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F83" s="234">
+        <v>1</v>
+      </c>
+      <c r="G83" s="234">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F84" s="234">
         <v>2</v>
       </c>
-      <c r="G82" s="1">
+      <c r="G84" s="234">
         <v>1.5</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C83" s="1" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E83" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F83" s="22">
+      <c r="E85" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="F85" s="4">
         <v>3</v>
       </c>
-      <c r="G83" s="22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C84" s="1" t="s">
+      <c r="G85" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="E86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F84" s="1">
-        <v>1</v>
-      </c>
-      <c r="G84" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C85" s="1" t="s">
+      <c r="F86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F85" s="1">
-        <v>2</v>
-      </c>
-      <c r="G85" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="D86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="E86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="F86" s="4">
-        <v>3</v>
-      </c>
-      <c r="G86" s="4">
-        <v>1</v>
+      <c r="G86" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G87" s="1">
-        <v>6</v>
+      <c r="B87" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
-        <v>50</v>
+      <c r="A88" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -76537,53 +76534,66 @@
       <c r="A90" t="s">
         <v>0</v>
       </c>
+      <c r="B90" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>0</v>
-      </c>
-      <c r="B91" t="s">
-        <v>1159</v>
-      </c>
+      <c r="B91" s="145" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C91" s="145"/>
+      <c r="D91" s="146"/>
+      <c r="E91" s="146"/>
+      <c r="F91" s="146"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B92" s="145" t="s">
-        <v>1160</v>
-      </c>
-      <c r="C92" s="145"/>
-      <c r="D92" s="146"/>
-      <c r="E92" s="146"/>
-      <c r="F92" s="146"/>
+      <c r="C92" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D92" s="229" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E92" s="147" t="s">
+        <v>1162</v>
+      </c>
+      <c r="F92" s="229" t="s">
+        <v>1166</v>
+      </c>
+      <c r="G92" s="148" t="s">
+        <v>1168</v>
+      </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C93" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D93" s="229" t="s">
-        <v>1161</v>
-      </c>
-      <c r="E93" s="147" t="s">
-        <v>1162</v>
-      </c>
-      <c r="F93" s="229" t="s">
-        <v>1166</v>
-      </c>
-      <c r="G93" s="148" t="s">
-        <v>1168</v>
+      <c r="C93" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D93" s="230" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F93" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G93" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C94" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D94" s="230" t="s">
-        <v>1164</v>
-      </c>
-      <c r="E94" s="1" t="s">
+      <c r="D94" s="232" t="str">
+        <f>D93</f>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F94" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G94" s="1">
         <v>1</v>
@@ -76594,17 +76604,17 @@
         <v>353</v>
       </c>
       <c r="D95" s="232" t="str">
-        <f>D94</f>
+        <f t="shared" ref="D95:D98" si="1">D94</f>
         <v>MPassInteg</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F95" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G95" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -76612,17 +76622,17 @@
         <v>353</v>
       </c>
       <c r="D96" s="232" t="str">
-        <f t="shared" ref="D96:D99" si="1">D95</f>
+        <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E96" s="6" t="s">
-        <v>1163</v>
+      <c r="E96" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F96" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G96" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="3:7" x14ac:dyDescent="0.25">
@@ -76633,67 +76643,67 @@
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E97" s="1" t="s">
+      <c r="E97" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F97" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G97" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C98" s="1" t="s">
+      <c r="C98" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D98" s="232" t="str">
+      <c r="D98" s="233" t="str">
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E98" s="6" t="s">
+      <c r="E98" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F98" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G98" s="1">
-        <v>1</v>
+      <c r="F98" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G98" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="99" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C99" s="22" t="s">
+      <c r="C99" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D99" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E99" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F99" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G99" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D99" s="230" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F99" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G99" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C100" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D100" s="230" t="s">
-        <v>1170</v>
-      </c>
-      <c r="E100" s="1" t="s">
+      <c r="D100" s="232" t="str">
+        <f>D99</f>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E100" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F100" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G100" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.25">
@@ -76701,17 +76711,17 @@
         <v>353</v>
       </c>
       <c r="D101" s="232" t="str">
-        <f>D100</f>
+        <f t="shared" ref="D101:D104" si="2">D100</f>
         <v>SPassPrim-PrimTank</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F101" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G101" s="1">
-        <v>1</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="102" spans="3:7" x14ac:dyDescent="0.25">
@@ -76719,17 +76729,17 @@
         <v>353</v>
       </c>
       <c r="D102" s="232" t="str">
-        <f t="shared" ref="D102:D105" si="2">D101</f>
+        <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E102" s="6" t="s">
-        <v>1163</v>
+      <c r="E102" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F102" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G102" s="1">
-        <v>1.1399999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="3:7" x14ac:dyDescent="0.25">
@@ -76740,67 +76750,67 @@
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E103" s="1" t="s">
+      <c r="E103" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F103" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G103" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C104" s="1" t="s">
+      <c r="C104" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D104" s="232" t="str">
+      <c r="D104" s="233" t="str">
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="E104" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F104" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G104" s="1">
-        <v>1</v>
+      <c r="F104" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G104" s="22">
+        <v>1.0900000000000001</v>
       </c>
     </row>
     <row r="105" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C105" s="22" t="s">
+      <c r="C105" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D105" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E105" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F105" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G105" s="22">
-        <v>1.0900000000000001</v>
+      <c r="D105" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F105" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G105" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C106" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D106" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="E106" s="1" t="s">
+      <c r="D106" s="232" t="str">
+        <f>D105</f>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E106" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F106" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G106" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.25">
@@ -76808,17 +76818,17 @@
         <v>353</v>
       </c>
       <c r="D107" s="232" t="str">
-        <f>D106</f>
+        <f t="shared" ref="D107:D110" si="3">D106</f>
         <v>MPassPrim-PrimTank</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F107" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G107" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.25">
@@ -76826,17 +76836,17 @@
         <v>353</v>
       </c>
       <c r="D108" s="232" t="str">
-        <f t="shared" ref="D108:D111" si="3">D107</f>
+        <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E108" s="6" t="s">
-        <v>1163</v>
+      <c r="E108" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F108" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G108" s="1">
-        <v>1.1499999999999999</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.25">
@@ -76847,67 +76857,67 @@
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="E109" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F109" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G109" s="1">
-        <v>0.98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C110" s="1" t="s">
+      <c r="C110" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D110" s="232" t="str">
+      <c r="D110" s="233" t="str">
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E110" s="6" t="s">
+      <c r="E110" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F110" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G110" s="1">
-        <v>1</v>
+      <c r="F110" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G110" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C111" s="22" t="s">
+      <c r="C111" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D111" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E111" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F111" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G111" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D111" s="230" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F111" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G111" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C112" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D112" s="230" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E112" s="1" t="s">
+      <c r="D112" s="232" t="str">
+        <f>D111</f>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E112" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F112" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G112" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -76915,17 +76925,17 @@
         <v>353</v>
       </c>
       <c r="D113" s="232" t="str">
-        <f>D112</f>
+        <f t="shared" ref="D113:D116" si="4">D112</f>
         <v>SPassPrim-SResist</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F113" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G113" s="1">
-        <v>1</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -76933,17 +76943,17 @@
         <v>353</v>
       </c>
       <c r="D114" s="232" t="str">
-        <f t="shared" ref="D114:D117" si="4">D113</f>
+        <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E114" s="6" t="s">
-        <v>1163</v>
+      <c r="E114" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F114" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G114" s="1">
-        <v>1.08</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -76954,67 +76964,67 @@
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E115" s="1" t="s">
+      <c r="E115" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F115" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G115" s="1">
-        <v>0.99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C116" s="1" t="s">
+      <c r="C116" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D116" s="232" t="str">
+      <c r="D116" s="233" t="str">
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E116" s="6" t="s">
+      <c r="E116" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F116" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G116" s="1">
-        <v>1</v>
+      <c r="F116" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G116" s="22">
+        <v>1.05</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C117" s="22" t="s">
+      <c r="C117" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D117" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E117" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F117" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G117" s="22">
-        <v>1.05</v>
+      <c r="D117" s="230" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F117" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G117" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D118" s="230" t="s">
-        <v>1173</v>
-      </c>
-      <c r="E118" s="1" t="s">
+      <c r="D118" s="232" t="str">
+        <f>D117</f>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F118" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G118" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -77022,17 +77032,17 @@
         <v>353</v>
       </c>
       <c r="D119" s="232" t="str">
-        <f>D118</f>
+        <f t="shared" ref="D119:D122" si="5">D118</f>
         <v>SPassPrim-Parallel</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F119" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G119" s="1">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -77040,17 +77050,17 @@
         <v>353</v>
       </c>
       <c r="D120" s="232" t="str">
-        <f t="shared" ref="D120:D123" si="5">D119</f>
+        <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E120" s="6" t="s">
-        <v>1163</v>
+      <c r="E120" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F120" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G120" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -77061,76 +77071,58 @@
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E121" s="1" t="s">
+      <c r="E121" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F121" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G121" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C122" s="1" t="s">
+      <c r="C122" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D122" s="232" t="str">
+      <c r="D122" s="233" t="str">
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E122" s="6" t="s">
+      <c r="E122" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F122" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G122" s="1">
-        <v>1</v>
+      <c r="F122" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G122" s="22">
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C123" s="22" t="s">
+      <c r="C123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D123" s="233" t="str">
-        <f t="shared" si="5"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E123" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F123" s="231" t="s">
+      <c r="D123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G123" s="22">
-        <v>1.1000000000000001</v>
+      <c r="E123" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F123" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G123" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F124" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G124" s="1">
-        <v>1</v>
+      <c r="B124" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="A125" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MF Central DHW branch pipe diam, Res Air2Wtr HP fixes and rule version ID updates for RC
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FEEA15-8B92-4F66-9DC4-44DB8FFB9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330A60BE-61FF-4FCF-8636-1F7798A2CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1170" windowWidth="20535" windowHeight="14760" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5910" yWindow="1080" windowWidth="17145" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8116" uniqueCount="1183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8118" uniqueCount="1184">
   <si>
     <t>;</t>
   </si>
@@ -3805,6 +3805,9 @@
   </si>
   <si>
     <t>SegIdx</t>
+  </si>
+  <si>
+    <t>08/26/26 - SAC - updated T24RDHW_LoopPipeSize table 2025+ Branch pipe diam from 1.5 (old value) to 0.75 for consistency w/ ACM AppB (dev #943)</t>
   </si>
 </sst>
 </file>
@@ -4488,7 +4491,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="235">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5025,9 +5028,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75206,7 +75206,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.85546875" customWidth="1"/>
@@ -75258,7 +75258,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>1176</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75266,63 +75266,60 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>1174</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
+      <c r="D7" t="s">
+        <v>1174</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
-      <c r="B8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>494</v>
-      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
-      <c r="B10" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
-      <c r="B12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>495</v>
-      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
-      <c r="C13">
-        <v>1</v>
+      <c r="B13" t="s">
+        <v>6</v>
       </c>
       <c r="D13" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -75330,10 +75327,10 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>1180</v>
+        <v>496</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -75341,10 +75338,10 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D15" t="s">
-        <v>497</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -75352,16 +75349,22 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="s">
-        <v>1181</v>
+        <v>497</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1181</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -75372,105 +75375,92 @@
       <c r="A19" t="s">
         <v>0</v>
       </c>
-      <c r="B19" t="s">
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B20" s="145" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="145" t="s">
         <v>544</v>
       </c>
-      <c r="C20" s="145"/>
-      <c r="D20" s="146"/>
-      <c r="E20" s="146"/>
-      <c r="F20" s="146"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="147" t="s">
+      <c r="C21" s="145"/>
+      <c r="D21" s="146"/>
+      <c r="E21" s="146"/>
+      <c r="F21" s="146"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C22" s="147" t="s">
         <v>433</v>
       </c>
-      <c r="D21" s="147" t="s">
+      <c r="D22" s="147" t="s">
         <v>1177</v>
       </c>
-      <c r="E21" s="147" t="s">
+      <c r="E22" s="147" t="s">
         <v>498</v>
       </c>
-      <c r="F21" s="147" t="s">
+      <c r="F22" s="147" t="s">
         <v>1182</v>
       </c>
-      <c r="G21" s="147" t="s">
+      <c r="G22" s="147" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="1" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C23" s="1" t="s">
         <v>1175</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E22" s="28" t="s">
-        <v>501</v>
-      </c>
-      <c r="F22" s="28">
-        <v>0</v>
-      </c>
-      <c r="G22" s="28">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="6" t="str">
-        <f>C22</f>
-        <v>&lt;2024</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="28" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G23" s="1">
-        <v>1</v>
+      <c r="F23" s="28">
+        <v>0</v>
+      </c>
+      <c r="G23" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="6" t="str">
-        <f t="shared" ref="C24:C30" si="0">C23</f>
+        <f>C23</f>
         <v>&lt;2024</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G24" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C25" s="6" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C25:C31" si="0">C24</f>
         <v>&lt;2024</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G25" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -75482,13 +75472,13 @@
         <v>353</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G26" s="1">
-        <v>2.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -75500,13 +75490,13 @@
         <v>353</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G27" s="1">
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -75518,13 +75508,13 @@
         <v>353</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G28" s="1">
-        <v>3.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -75536,65 +75526,66 @@
         <v>353</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G29" s="1">
-        <v>4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="36" t="str">
+      <c r="C30" s="6" t="str">
         <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G30" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31" s="36" t="str">
+        <f t="shared" si="0"/>
+        <v>&lt;2024</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F31" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="G30" s="4">
+      <c r="G31" s="4">
         <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E31" s="28" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F31" s="28">
-        <v>0</v>
-      </c>
-      <c r="G31" s="28">
-        <v>1.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D32" s="1">
-        <v>0</v>
-      </c>
-      <c r="E32" s="1" t="s">
+      <c r="D32" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E32" s="28" t="s">
         <v>1178</v>
       </c>
-      <c r="F32" s="1">
-        <v>1</v>
-      </c>
-      <c r="G32" s="1">
-        <v>1</v>
+      <c r="F32" s="28">
+        <v>0</v>
+      </c>
+      <c r="G32" s="28">
+        <v>0.75</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
@@ -75608,10 +75599,10 @@
         <v>1178</v>
       </c>
       <c r="F33" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="1">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.25">
@@ -75621,13 +75612,13 @@
       <c r="D34" s="1">
         <v>0</v>
       </c>
-      <c r="E34" s="22" t="s">
+      <c r="E34" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="F34" s="22">
-        <v>3</v>
-      </c>
-      <c r="G34" s="22">
+      <c r="F34" s="1">
+        <v>2</v>
+      </c>
+      <c r="G34" s="1">
         <v>0.75</v>
       </c>
     </row>
@@ -75638,14 +75629,14 @@
       <c r="D35" s="1">
         <v>0</v>
       </c>
-      <c r="E35" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="F35" s="1">
-        <v>1</v>
-      </c>
-      <c r="G35" s="1">
-        <v>1.5</v>
+      <c r="E35" s="22" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F35" s="22">
+        <v>3</v>
+      </c>
+      <c r="G35" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
@@ -75659,10 +75650,10 @@
         <v>502</v>
       </c>
       <c r="F36" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.25">
@@ -75672,14 +75663,14 @@
       <c r="D37" s="1">
         <v>0</v>
       </c>
-      <c r="E37" s="22" t="s">
+      <c r="E37" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="F37" s="22">
-        <v>3</v>
-      </c>
-      <c r="G37" s="22">
-        <v>0.75</v>
+      <c r="F37" s="1">
+        <v>2</v>
+      </c>
+      <c r="G37" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
@@ -75689,14 +75680,14 @@
       <c r="D38" s="1">
         <v>0</v>
       </c>
-      <c r="E38" s="1" t="s">
-        <v>503</v>
-      </c>
-      <c r="F38" s="1">
-        <v>1</v>
-      </c>
-      <c r="G38" s="1">
-        <v>2</v>
+      <c r="E38" s="22" t="s">
+        <v>502</v>
+      </c>
+      <c r="F38" s="22">
+        <v>3</v>
+      </c>
+      <c r="G38" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
@@ -75710,10 +75701,10 @@
         <v>503</v>
       </c>
       <c r="F39" s="1">
+        <v>1</v>
+      </c>
+      <c r="G39" s="1">
         <v>2</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1.5</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
@@ -75723,13 +75714,13 @@
       <c r="D40" s="1">
         <v>0</v>
       </c>
-      <c r="E40" s="22" t="s">
+      <c r="E40" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="F40" s="22">
-        <v>3</v>
-      </c>
-      <c r="G40" s="22">
+      <c r="F40" s="1">
+        <v>2</v>
+      </c>
+      <c r="G40" s="1">
         <v>1.5</v>
       </c>
     </row>
@@ -75740,14 +75731,14 @@
       <c r="D41" s="1">
         <v>0</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F41" s="1">
-        <v>1</v>
-      </c>
-      <c r="G41" s="1">
-        <v>2.5</v>
+      <c r="E41" s="22" t="s">
+        <v>503</v>
+      </c>
+      <c r="F41" s="22">
+        <v>3</v>
+      </c>
+      <c r="G41" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="42" spans="3:7" x14ac:dyDescent="0.25">
@@ -75761,10 +75752,10 @@
         <v>1179</v>
       </c>
       <c r="F42" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G42" s="1">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.25">
@@ -75774,13 +75765,13 @@
       <c r="D43" s="1">
         <v>0</v>
       </c>
-      <c r="E43" s="22" t="s">
+      <c r="E43" s="1" t="s">
         <v>1179</v>
       </c>
-      <c r="F43" s="22">
-        <v>3</v>
-      </c>
-      <c r="G43" s="22">
+      <c r="F43" s="1">
+        <v>2</v>
+      </c>
+      <c r="G43" s="1">
         <v>1.5</v>
       </c>
     </row>
@@ -75791,14 +75782,14 @@
       <c r="D44" s="1">
         <v>0</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="F44" s="1">
-        <v>1</v>
-      </c>
-      <c r="G44" s="1">
+      <c r="E44" s="22" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F44" s="22">
         <v>3</v>
+      </c>
+      <c r="G44" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="45" spans="3:7" x14ac:dyDescent="0.25">
@@ -75812,10 +75803,10 @@
         <v>505</v>
       </c>
       <c r="F45" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" s="1">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46" spans="3:7" x14ac:dyDescent="0.25">
@@ -75825,13 +75816,13 @@
       <c r="D46" s="1">
         <v>0</v>
       </c>
-      <c r="E46" s="22" t="s">
+      <c r="E46" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="F46" s="22">
-        <v>3</v>
-      </c>
-      <c r="G46" s="22">
+      <c r="F46" s="1">
+        <v>2</v>
+      </c>
+      <c r="G46" s="1">
         <v>1.5</v>
       </c>
     </row>
@@ -75842,14 +75833,14 @@
       <c r="D47" s="1">
         <v>0</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F47" s="1">
-        <v>1</v>
-      </c>
-      <c r="G47" s="1">
-        <v>3.5</v>
+      <c r="E47" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="F47" s="22">
+        <v>3</v>
+      </c>
+      <c r="G47" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.25">
@@ -75863,10 +75854,10 @@
         <v>506</v>
       </c>
       <c r="F48" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" s="1">
-        <v>2</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="49" spans="3:7" x14ac:dyDescent="0.25">
@@ -75876,14 +75867,14 @@
       <c r="D49" s="1">
         <v>0</v>
       </c>
-      <c r="E49" s="22" t="s">
+      <c r="E49" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="F49" s="22">
-        <v>3</v>
-      </c>
-      <c r="G49" s="22">
-        <v>1.5</v>
+      <c r="F49" s="1">
+        <v>2</v>
+      </c>
+      <c r="G49" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="3:7" x14ac:dyDescent="0.25">
@@ -75893,14 +75884,14 @@
       <c r="D50" s="1">
         <v>0</v>
       </c>
-      <c r="E50" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="F50" s="1">
-        <v>1</v>
-      </c>
-      <c r="G50" s="1">
-        <v>4</v>
+      <c r="E50" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="F50" s="22">
+        <v>3</v>
+      </c>
+      <c r="G50" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="51" spans="3:7" x14ac:dyDescent="0.25">
@@ -75914,10 +75905,10 @@
         <v>507</v>
       </c>
       <c r="F51" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="3:7" x14ac:dyDescent="0.25">
@@ -75927,14 +75918,14 @@
       <c r="D52" s="1">
         <v>0</v>
       </c>
-      <c r="E52" s="22" t="s">
+      <c r="E52" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="F52" s="22">
-        <v>3</v>
-      </c>
-      <c r="G52" s="22">
-        <v>1.5</v>
+      <c r="F52" s="1">
+        <v>2</v>
+      </c>
+      <c r="G52" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="3:7" x14ac:dyDescent="0.25">
@@ -75944,14 +75935,14 @@
       <c r="D53" s="1">
         <v>0</v>
       </c>
-      <c r="E53" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="F53" s="1">
-        <v>1</v>
-      </c>
-      <c r="G53" s="1">
-        <v>5</v>
+      <c r="E53" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="F53" s="22">
+        <v>3</v>
+      </c>
+      <c r="G53" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="54" spans="3:7" x14ac:dyDescent="0.25">
@@ -75965,10 +75956,10 @@
         <v>508</v>
       </c>
       <c r="F54" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G54" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" spans="3:7" x14ac:dyDescent="0.25">
@@ -75978,82 +75969,82 @@
       <c r="D55" s="1">
         <v>0</v>
       </c>
-      <c r="E55" s="22" t="s">
+      <c r="E55" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="F55" s="22">
+      <c r="F55" s="1">
+        <v>2</v>
+      </c>
+      <c r="G55" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D56" s="1">
+        <v>0</v>
+      </c>
+      <c r="E56" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="F56" s="22">
         <v>3</v>
       </c>
-      <c r="G55" s="22">
+      <c r="G56" s="22">
         <v>1.5</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="234" t="s">
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D56" s="234">
-        <v>0</v>
-      </c>
-      <c r="E56" s="234" t="s">
+      <c r="D57" s="1">
+        <v>0</v>
+      </c>
+      <c r="E57" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F56" s="234">
-        <v>1</v>
-      </c>
-      <c r="G56" s="234">
+      <c r="F57" s="1">
+        <v>1</v>
+      </c>
+      <c r="G57" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="234" t="s">
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D57" s="234">
-        <v>0</v>
-      </c>
-      <c r="E57" s="234" t="s">
+      <c r="D58" s="1">
+        <v>0</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F57" s="234">
+      <c r="F58" s="1">
         <v>2</v>
       </c>
-      <c r="G57" s="234">
+      <c r="G58" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="22" t="s">
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D58" s="22">
-        <v>0</v>
-      </c>
-      <c r="E58" s="22" t="s">
+      <c r="D59" s="22">
+        <v>0</v>
+      </c>
+      <c r="E59" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="F58" s="22">
+      <c r="F59" s="22">
         <v>3</v>
       </c>
-      <c r="G58" s="22">
+      <c r="G59" s="22">
         <v>1.5</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F59" s="1">
-        <v>1</v>
-      </c>
-      <c r="G59" s="1">
-        <v>1</v>
       </c>
     </row>
     <row r="60" spans="3:7" x14ac:dyDescent="0.25">
@@ -76067,10 +76058,10 @@
         <v>1178</v>
       </c>
       <c r="F60" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60" s="1">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="3:7" x14ac:dyDescent="0.25">
@@ -76080,13 +76071,13 @@
       <c r="D61" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E61" s="22" t="s">
+      <c r="E61" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="F61" s="22">
-        <v>3</v>
-      </c>
-      <c r="G61" s="22">
+      <c r="F61" s="1">
+        <v>2</v>
+      </c>
+      <c r="G61" s="1">
         <v>0.75</v>
       </c>
     </row>
@@ -76097,14 +76088,14 @@
       <c r="D62" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E62" s="1" t="s">
-        <v>502</v>
-      </c>
-      <c r="F62" s="1">
-        <v>1</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.5</v>
+      <c r="E62" s="22" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F62" s="22">
+        <v>3</v>
+      </c>
+      <c r="G62" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="63" spans="3:7" x14ac:dyDescent="0.25">
@@ -76118,10 +76109,10 @@
         <v>502</v>
       </c>
       <c r="F63" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="64" spans="3:7" x14ac:dyDescent="0.25">
@@ -76131,14 +76122,14 @@
       <c r="D64" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E64" s="22" t="s">
+      <c r="E64" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="F64" s="22">
-        <v>3</v>
-      </c>
-      <c r="G64" s="22">
-        <v>0.75</v>
+      <c r="F64" s="1">
+        <v>2</v>
+      </c>
+      <c r="G64" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="65" spans="3:7" x14ac:dyDescent="0.25">
@@ -76148,14 +76139,14 @@
       <c r="D65" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>503</v>
-      </c>
-      <c r="F65" s="1">
-        <v>1</v>
-      </c>
-      <c r="G65" s="1">
-        <v>1.5</v>
+      <c r="E65" s="22" t="s">
+        <v>502</v>
+      </c>
+      <c r="F65" s="22">
+        <v>3</v>
+      </c>
+      <c r="G65" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="66" spans="3:7" x14ac:dyDescent="0.25">
@@ -76169,7 +76160,7 @@
         <v>503</v>
       </c>
       <c r="F66" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G66" s="1">
         <v>1.5</v>
@@ -76182,14 +76173,14 @@
       <c r="D67" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E67" s="22" t="s">
+      <c r="E67" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="F67" s="22">
-        <v>3</v>
-      </c>
-      <c r="G67" s="22">
-        <v>1</v>
+      <c r="F67" s="1">
+        <v>2</v>
+      </c>
+      <c r="G67" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -76199,14 +76190,14 @@
       <c r="D68" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E68" s="1" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F68" s="1">
-        <v>1</v>
-      </c>
-      <c r="G68" s="1">
-        <v>1.5</v>
+      <c r="E68" s="22" t="s">
+        <v>503</v>
+      </c>
+      <c r="F68" s="22">
+        <v>3</v>
+      </c>
+      <c r="G68" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="3:7" x14ac:dyDescent="0.25">
@@ -76220,7 +76211,7 @@
         <v>1179</v>
       </c>
       <c r="F69" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G69" s="1">
         <v>1.5</v>
@@ -76233,14 +76224,14 @@
       <c r="D70" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E70" s="22" t="s">
+      <c r="E70" s="1" t="s">
         <v>1179</v>
       </c>
-      <c r="F70" s="22">
-        <v>3</v>
-      </c>
-      <c r="G70" s="22">
-        <v>1</v>
+      <c r="F70" s="1">
+        <v>2</v>
+      </c>
+      <c r="G70" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="71" spans="3:7" x14ac:dyDescent="0.25">
@@ -76250,14 +76241,14 @@
       <c r="D71" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E71" s="1" t="s">
-        <v>505</v>
-      </c>
-      <c r="F71" s="1">
-        <v>1</v>
-      </c>
-      <c r="G71" s="1">
-        <v>2</v>
+      <c r="E71" s="22" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F71" s="22">
+        <v>3</v>
+      </c>
+      <c r="G71" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="3:7" x14ac:dyDescent="0.25">
@@ -76271,10 +76262,10 @@
         <v>505</v>
       </c>
       <c r="F72" s="1">
+        <v>1</v>
+      </c>
+      <c r="G72" s="1">
         <v>2</v>
-      </c>
-      <c r="G72" s="1">
-        <v>1.5</v>
       </c>
     </row>
     <row r="73" spans="3:7" x14ac:dyDescent="0.25">
@@ -76284,14 +76275,14 @@
       <c r="D73" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E73" s="22" t="s">
+      <c r="E73" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="F73" s="22">
-        <v>3</v>
-      </c>
-      <c r="G73" s="22">
-        <v>1</v>
+      <c r="F73" s="1">
+        <v>2</v>
+      </c>
+      <c r="G73" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="74" spans="3:7" x14ac:dyDescent="0.25">
@@ -76301,14 +76292,14 @@
       <c r="D74" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E74" s="1" t="s">
-        <v>506</v>
-      </c>
-      <c r="F74" s="1">
-        <v>1</v>
-      </c>
-      <c r="G74" s="1">
+      <c r="E74" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="F74" s="22">
         <v>3</v>
+      </c>
+      <c r="G74" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="3:7" x14ac:dyDescent="0.25">
@@ -76322,10 +76313,10 @@
         <v>506</v>
       </c>
       <c r="F75" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G75" s="1">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76" spans="3:7" x14ac:dyDescent="0.25">
@@ -76335,14 +76326,14 @@
       <c r="D76" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E76" s="22" t="s">
+      <c r="E76" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="F76" s="22">
-        <v>3</v>
-      </c>
-      <c r="G76" s="22">
-        <v>1</v>
+      <c r="F76" s="1">
+        <v>2</v>
+      </c>
+      <c r="G76" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="77" spans="3:7" x14ac:dyDescent="0.25">
@@ -76352,14 +76343,14 @@
       <c r="D77" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E77" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="F77" s="1">
-        <v>1</v>
-      </c>
-      <c r="G77" s="1">
+      <c r="E77" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="F77" s="22">
         <v>3</v>
+      </c>
+      <c r="G77" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="3:7" x14ac:dyDescent="0.25">
@@ -76373,10 +76364,10 @@
         <v>507</v>
       </c>
       <c r="F78" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G78" s="1">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="79" spans="3:7" x14ac:dyDescent="0.25">
@@ -76386,14 +76377,14 @@
       <c r="D79" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E79" s="22" t="s">
+      <c r="E79" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="F79" s="22">
-        <v>3</v>
-      </c>
-      <c r="G79" s="22">
-        <v>1</v>
+      <c r="F79" s="1">
+        <v>2</v>
+      </c>
+      <c r="G79" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="80" spans="3:7" x14ac:dyDescent="0.25">
@@ -76403,14 +76394,14 @@
       <c r="D80" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E80" s="1" t="s">
-        <v>508</v>
-      </c>
-      <c r="F80" s="1">
-        <v>1</v>
-      </c>
-      <c r="G80" s="1">
+      <c r="E80" s="22" t="s">
+        <v>507</v>
+      </c>
+      <c r="F80" s="22">
         <v>3</v>
+      </c>
+      <c r="G80" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -76424,10 +76415,10 @@
         <v>508</v>
       </c>
       <c r="F81" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G81" s="1">
-        <v>1.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -76437,92 +76428,104 @@
       <c r="D82" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E82" s="22" t="s">
+      <c r="E82" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="F82" s="22">
+      <c r="F82" s="1">
+        <v>2</v>
+      </c>
+      <c r="G82" s="1">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C83" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E83" s="22" t="s">
+        <v>508</v>
+      </c>
+      <c r="F83" s="22">
         <v>3</v>
       </c>
-      <c r="G82" s="22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C83" s="234" t="s">
+      <c r="G83" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C84" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D83" s="234" t="s">
+      <c r="D84" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E83" s="234" t="s">
+      <c r="E84" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F83" s="234">
-        <v>1</v>
-      </c>
-      <c r="G83" s="234">
+      <c r="F84" s="1">
+        <v>1</v>
+      </c>
+      <c r="G84" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C84" s="234" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C85" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D84" s="234" t="s">
+      <c r="D85" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E84" s="234" t="s">
+      <c r="E85" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F84" s="234">
+      <c r="F85" s="1">
         <v>2</v>
       </c>
-      <c r="G84" s="234">
+      <c r="G85" s="1">
         <v>1.5</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C85" s="4" t="s">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C86" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="D85" s="4" t="s">
+      <c r="D86" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E85" s="4" t="s">
+      <c r="E86" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="F85" s="4">
+      <c r="F86" s="4">
         <v>3</v>
       </c>
-      <c r="G85" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C86" s="1" t="s">
+      <c r="G86" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C87" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D86" s="1" t="s">
+      <c r="D87" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E86" s="1" t="s">
+      <c r="E87" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F86" s="1" t="s">
+      <c r="F87" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G86" s="1">
+      <c r="G87" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B87" t="s">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B88" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -76534,66 +76537,53 @@
       <c r="A90" t="s">
         <v>0</v>
       </c>
-      <c r="B90" t="s">
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B91" t="s">
         <v>1159</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B91" s="145" t="s">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B92" s="145" t="s">
         <v>1160</v>
       </c>
-      <c r="C91" s="145"/>
-      <c r="D91" s="146"/>
-      <c r="E91" s="146"/>
-      <c r="F91" s="146"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C92" s="147" t="s">
+      <c r="C92" s="145"/>
+      <c r="D92" s="146"/>
+      <c r="E92" s="146"/>
+      <c r="F92" s="146"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C93" s="147" t="s">
         <v>433</v>
       </c>
-      <c r="D92" s="229" t="s">
+      <c r="D93" s="229" t="s">
         <v>1161</v>
       </c>
-      <c r="E92" s="147" t="s">
+      <c r="E93" s="147" t="s">
         <v>1162</v>
       </c>
-      <c r="F92" s="229" t="s">
+      <c r="F93" s="229" t="s">
         <v>1166</v>
       </c>
-      <c r="G92" s="148" t="s">
+      <c r="G93" s="148" t="s">
         <v>1168</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C93" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D93" s="230" t="s">
-        <v>1164</v>
-      </c>
-      <c r="E93" s="1" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F93" s="230" t="s">
-        <v>1165</v>
-      </c>
-      <c r="G93" s="1">
-        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C94" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D94" s="232" t="str">
-        <f>D93</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E94" s="6" t="s">
+      <c r="D94" s="230" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E94" s="1" t="s">
         <v>1163</v>
       </c>
       <c r="F94" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G94" s="1">
         <v>1</v>
@@ -76604,17 +76594,17 @@
         <v>353</v>
       </c>
       <c r="D95" s="232" t="str">
-        <f t="shared" ref="D95:D98" si="1">D94</f>
+        <f>D94</f>
         <v>MPassInteg</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F95" s="230" t="s">
-        <v>353</v>
+        <v>1167</v>
       </c>
       <c r="G95" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -76622,17 +76612,17 @@
         <v>353</v>
       </c>
       <c r="D96" s="232" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D96:D99" si="1">D95</f>
         <v>MPassInteg</v>
       </c>
-      <c r="E96" s="1" t="s">
-        <v>1169</v>
+      <c r="E96" s="6" t="s">
+        <v>1163</v>
       </c>
       <c r="F96" s="230" t="s">
-        <v>1165</v>
+        <v>353</v>
       </c>
       <c r="G96" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="97" spans="3:7" x14ac:dyDescent="0.25">
@@ -76643,67 +76633,67 @@
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E97" s="6" t="s">
+      <c r="E97" s="1" t="s">
         <v>1169</v>
       </c>
       <c r="F97" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G97" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C98" s="22" t="s">
+      <c r="C98" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D98" s="233" t="str">
+      <c r="D98" s="232" t="str">
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E98" s="113" t="s">
+      <c r="E98" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="F98" s="231" t="s">
+      <c r="F98" s="230" t="s">
+        <v>1167</v>
+      </c>
+      <c r="G98" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C99" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G98" s="22">
+      <c r="D99" s="233" t="str">
+        <f t="shared" si="1"/>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E99" s="113" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F99" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G99" s="22">
         <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C99" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D99" s="230" t="s">
-        <v>1170</v>
-      </c>
-      <c r="E99" s="1" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F99" s="230" t="s">
-        <v>1165</v>
-      </c>
-      <c r="G99" s="1">
-        <v>0.96</v>
       </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C100" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D100" s="232" t="str">
-        <f>D99</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E100" s="6" t="s">
+      <c r="D100" s="230" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E100" s="1" t="s">
         <v>1163</v>
       </c>
       <c r="F100" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G100" s="1">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.25">
@@ -76711,17 +76701,17 @@
         <v>353</v>
       </c>
       <c r="D101" s="232" t="str">
-        <f t="shared" ref="D101:D104" si="2">D100</f>
+        <f>D100</f>
         <v>SPassPrim-PrimTank</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F101" s="230" t="s">
-        <v>353</v>
+        <v>1167</v>
       </c>
       <c r="G101" s="1">
-        <v>1.1399999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102" spans="3:7" x14ac:dyDescent="0.25">
@@ -76729,17 +76719,17 @@
         <v>353</v>
       </c>
       <c r="D102" s="232" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D102:D105" si="2">D101</f>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E102" s="1" t="s">
-        <v>1169</v>
+      <c r="E102" s="6" t="s">
+        <v>1163</v>
       </c>
       <c r="F102" s="230" t="s">
-        <v>1165</v>
+        <v>353</v>
       </c>
       <c r="G102" s="1">
-        <v>1</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="103" spans="3:7" x14ac:dyDescent="0.25">
@@ -76750,67 +76740,67 @@
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E103" s="6" t="s">
+      <c r="E103" s="1" t="s">
         <v>1169</v>
       </c>
       <c r="F103" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G103" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C104" s="22" t="s">
+      <c r="C104" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D104" s="233" t="str">
+      <c r="D104" s="232" t="str">
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E104" s="113" t="s">
+      <c r="E104" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="F104" s="231" t="s">
+      <c r="F104" s="230" t="s">
+        <v>1167</v>
+      </c>
+      <c r="G104" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C105" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G104" s="22">
+      <c r="D105" s="233" t="str">
+        <f t="shared" si="2"/>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E105" s="113" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F105" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G105" s="22">
         <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C105" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D105" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="E105" s="1" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F105" s="230" t="s">
-        <v>1165</v>
-      </c>
-      <c r="G105" s="1">
-        <v>0.96</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C106" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D106" s="232" t="str">
-        <f>D105</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E106" s="6" t="s">
+      <c r="D106" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E106" s="1" t="s">
         <v>1163</v>
       </c>
       <c r="F106" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G106" s="1">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.25">
@@ -76818,17 +76808,17 @@
         <v>353</v>
       </c>
       <c r="D107" s="232" t="str">
-        <f t="shared" ref="D107:D110" si="3">D106</f>
+        <f>D106</f>
         <v>MPassPrim-PrimTank</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F107" s="230" t="s">
-        <v>353</v>
+        <v>1167</v>
       </c>
       <c r="G107" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.25">
@@ -76836,17 +76826,17 @@
         <v>353</v>
       </c>
       <c r="D108" s="232" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D108:D111" si="3">D107</f>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E108" s="1" t="s">
-        <v>1169</v>
+      <c r="E108" s="6" t="s">
+        <v>1163</v>
       </c>
       <c r="F108" s="230" t="s">
-        <v>1165</v>
+        <v>353</v>
       </c>
       <c r="G108" s="1">
-        <v>0.98</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.25">
@@ -76857,67 +76847,67 @@
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E109" s="6" t="s">
+      <c r="E109" s="1" t="s">
         <v>1169</v>
       </c>
       <c r="F109" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G109" s="1">
-        <v>1</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C110" s="22" t="s">
+      <c r="C110" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D110" s="233" t="str">
+      <c r="D110" s="232" t="str">
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E110" s="113" t="s">
+      <c r="E110" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="F110" s="231" t="s">
+      <c r="F110" s="230" t="s">
+        <v>1167</v>
+      </c>
+      <c r="G110" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C111" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G110" s="22">
+      <c r="D111" s="233" t="str">
+        <f t="shared" si="3"/>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E111" s="113" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F111" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G111" s="22">
         <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C111" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D111" s="230" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E111" s="1" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F111" s="230" t="s">
-        <v>1165</v>
-      </c>
-      <c r="G111" s="1">
-        <v>0.96</v>
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C112" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D112" s="232" t="str">
-        <f>D111</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E112" s="6" t="s">
+      <c r="D112" s="230" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E112" s="1" t="s">
         <v>1163</v>
       </c>
       <c r="F112" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G112" s="1">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -76925,17 +76915,17 @@
         <v>353</v>
       </c>
       <c r="D113" s="232" t="str">
-        <f t="shared" ref="D113:D116" si="4">D112</f>
+        <f>D112</f>
         <v>SPassPrim-SResist</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F113" s="230" t="s">
-        <v>353</v>
+        <v>1167</v>
       </c>
       <c r="G113" s="1">
-        <v>1.08</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -76943,17 +76933,17 @@
         <v>353</v>
       </c>
       <c r="D114" s="232" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="D114:D117" si="4">D113</f>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E114" s="1" t="s">
-        <v>1169</v>
+      <c r="E114" s="6" t="s">
+        <v>1163</v>
       </c>
       <c r="F114" s="230" t="s">
-        <v>1165</v>
+        <v>353</v>
       </c>
       <c r="G114" s="1">
-        <v>0.99</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -76964,67 +76954,67 @@
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E115" s="6" t="s">
+      <c r="E115" s="1" t="s">
         <v>1169</v>
       </c>
       <c r="F115" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G115" s="1">
-        <v>1</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C116" s="22" t="s">
+      <c r="C116" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D116" s="233" t="str">
+      <c r="D116" s="232" t="str">
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E116" s="113" t="s">
+      <c r="E116" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="F116" s="231" t="s">
+      <c r="F116" s="230" t="s">
+        <v>1167</v>
+      </c>
+      <c r="G116" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C117" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G116" s="22">
+      <c r="D117" s="233" t="str">
+        <f t="shared" si="4"/>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E117" s="113" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F117" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G117" s="22">
         <v>1.05</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C117" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D117" s="230" t="s">
-        <v>1173</v>
-      </c>
-      <c r="E117" s="1" t="s">
-        <v>1163</v>
-      </c>
-      <c r="F117" s="230" t="s">
-        <v>1165</v>
-      </c>
-      <c r="G117" s="1">
-        <v>0.96</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D118" s="232" t="str">
-        <f>D117</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E118" s="6" t="s">
+      <c r="D118" s="230" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E118" s="1" t="s">
         <v>1163</v>
       </c>
       <c r="F118" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G118" s="1">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -77032,17 +77022,17 @@
         <v>353</v>
       </c>
       <c r="D119" s="232" t="str">
-        <f t="shared" ref="D119:D122" si="5">D118</f>
+        <f>D118</f>
         <v>SPassPrim-Parallel</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F119" s="230" t="s">
-        <v>353</v>
+        <v>1167</v>
       </c>
       <c r="G119" s="1">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -77050,17 +77040,17 @@
         <v>353</v>
       </c>
       <c r="D120" s="232" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D120:D123" si="5">D119</f>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E120" s="1" t="s">
-        <v>1169</v>
+      <c r="E120" s="6" t="s">
+        <v>1163</v>
       </c>
       <c r="F120" s="230" t="s">
-        <v>1165</v>
+        <v>353</v>
       </c>
       <c r="G120" s="1">
-        <v>0.96</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -77071,58 +77061,76 @@
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E121" s="6" t="s">
+      <c r="E121" s="1" t="s">
         <v>1169</v>
       </c>
       <c r="F121" s="230" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G121" s="1">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C122" s="22" t="s">
+      <c r="C122" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D122" s="233" t="str">
+      <c r="D122" s="232" t="str">
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E122" s="113" t="s">
+      <c r="E122" s="6" t="s">
         <v>1169</v>
       </c>
-      <c r="F122" s="231" t="s">
+      <c r="F122" s="230" t="s">
+        <v>1167</v>
+      </c>
+      <c r="G122" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C123" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="G122" s="22">
+      <c r="D123" s="233" t="str">
+        <f t="shared" si="5"/>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E123" s="113" t="s">
+        <v>1169</v>
+      </c>
+      <c r="F123" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G123" s="22">
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C123" s="1" t="s">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C124" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D123" s="1" t="s">
+      <c r="D124" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E123" s="1" t="s">
+      <c r="E124" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F123" s="230" t="s">
+      <c r="F124" s="230" t="s">
         <v>353</v>
       </c>
-      <c r="G123" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B124" t="s">
+      <c r="G124" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B125" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update rule to set DHW baseline to heat-pump for relocatable and permanent precheck school buildings
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330A60BE-61FF-4FCF-8636-1F7798A2CDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FEEA15-8B92-4F66-9DC4-44DB8FFB9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5910" yWindow="1080" windowWidth="17145" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1170" windowWidth="20535" windowHeight="14760" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8118" uniqueCount="1184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8116" uniqueCount="1183">
   <si>
     <t>;</t>
   </si>
@@ -3805,9 +3805,6 @@
   </si>
   <si>
     <t>SegIdx</t>
-  </si>
-  <si>
-    <t>08/26/26 - SAC - updated T24RDHW_LoopPipeSize table 2025+ Branch pipe diam from 1.5 (old value) to 0.75 for consistency w/ ACM AppB (dev #943)</t>
   </si>
 </sst>
 </file>
@@ -4491,7 +4488,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="235">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5028,6 +5025,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75206,7 +75206,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.85546875" customWidth="1"/>
@@ -75258,7 +75258,7 @@
         <v>3</v>
       </c>
       <c r="D5" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75266,60 +75266,63 @@
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
-      <c r="D7" t="s">
-        <v>1174</v>
-      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" t="s">
+        <v>494</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9" t="s">
-        <v>494</v>
-      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" t="s">
+        <v>495</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
-      <c r="B13" t="s">
-        <v>6</v>
+      <c r="C13">
+        <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -75327,10 +75330,10 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>496</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -75338,10 +75341,10 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D15" t="s">
-        <v>1180</v>
+        <v>497</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -75349,22 +75352,16 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="s">
-        <v>497</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17" t="s">
-        <v>1181</v>
-      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -75375,92 +75372,105 @@
       <c r="A19" t="s">
         <v>0</v>
       </c>
+      <c r="B19" t="s">
+        <v>500</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" t="s">
-        <v>500</v>
-      </c>
+      <c r="B20" s="145" t="s">
+        <v>544</v>
+      </c>
+      <c r="C20" s="145"/>
+      <c r="D20" s="146"/>
+      <c r="E20" s="146"/>
+      <c r="F20" s="146"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B21" s="145" t="s">
-        <v>544</v>
-      </c>
-      <c r="C21" s="145"/>
-      <c r="D21" s="146"/>
-      <c r="E21" s="146"/>
-      <c r="F21" s="146"/>
+      <c r="C21" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D21" s="147" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E21" s="147" t="s">
+        <v>498</v>
+      </c>
+      <c r="F21" s="147" t="s">
+        <v>1182</v>
+      </c>
+      <c r="G21" s="147" t="s">
+        <v>499</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D22" s="147" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E22" s="147" t="s">
-        <v>498</v>
-      </c>
-      <c r="F22" s="147" t="s">
-        <v>1182</v>
-      </c>
-      <c r="G22" s="147" t="s">
-        <v>499</v>
+      <c r="C22" s="1" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E22" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="F22" s="28">
+        <v>0</v>
+      </c>
+      <c r="G22" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="1" t="s">
-        <v>1175</v>
+      <c r="C23" s="6" t="str">
+        <f>C22</f>
+        <v>&lt;2024</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E23" s="28" t="s">
+      <c r="E23" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="28">
-        <v>0</v>
-      </c>
-      <c r="G23" s="28">
-        <v>1.5</v>
+      <c r="F23" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="G23" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="6" t="str">
-        <f>C23</f>
+        <f t="shared" ref="C24:C30" si="0">C23</f>
         <v>&lt;2024</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G24" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C25" s="6" t="str">
-        <f t="shared" ref="C25:C31" si="0">C24</f>
+        <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G25" s="1">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -75472,13 +75482,13 @@
         <v>353</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G26" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -75490,13 +75500,13 @@
         <v>353</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G27" s="1">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -75508,13 +75518,13 @@
         <v>353</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G28" s="1">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -75526,66 +75536,65 @@
         <v>353</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>353</v>
       </c>
       <c r="G29" s="1">
-        <v>3.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="6" t="str">
+      <c r="C30" s="36" t="str">
         <f t="shared" si="0"/>
         <v>&lt;2024</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>507</v>
-      </c>
-      <c r="F30" s="1" t="s">
+      <c r="E30" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="F30" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="G30" s="1">
-        <v>4</v>
+      <c r="G30" s="4">
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31" s="36" t="str">
-        <f t="shared" si="0"/>
-        <v>&lt;2024</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E31" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="F31" s="4" t="s">
+      <c r="D31" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G31" s="4">
-        <v>5</v>
+      <c r="E31" s="28" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F31" s="28">
+        <v>0</v>
+      </c>
+      <c r="G31" s="28">
+        <v>1.5</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E32" s="28" t="s">
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1" t="s">
         <v>1178</v>
       </c>
-      <c r="F32" s="28">
-        <v>0</v>
-      </c>
-      <c r="G32" s="28">
-        <v>0.75</v>
+      <c r="F32" s="1">
+        <v>1</v>
+      </c>
+      <c r="G32" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="3:7" x14ac:dyDescent="0.25">
@@ -75599,10 +75608,10 @@
         <v>1178</v>
       </c>
       <c r="F33" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34" spans="3:7" x14ac:dyDescent="0.25">
@@ -75612,13 +75621,13 @@
       <c r="D34" s="1">
         <v>0</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F34" s="1">
-        <v>2</v>
-      </c>
-      <c r="G34" s="1">
+      <c r="F34" s="22">
+        <v>3</v>
+      </c>
+      <c r="G34" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -75629,14 +75638,14 @@
       <c r="D35" s="1">
         <v>0</v>
       </c>
-      <c r="E35" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F35" s="22">
-        <v>3</v>
-      </c>
-      <c r="G35" s="22">
-        <v>0.75</v>
+      <c r="E35" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F35" s="1">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="36" spans="3:7" x14ac:dyDescent="0.25">
@@ -75650,10 +75659,10 @@
         <v>502</v>
       </c>
       <c r="F36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="3:7" x14ac:dyDescent="0.25">
@@ -75663,14 +75672,14 @@
       <c r="D37" s="1">
         <v>0</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F37" s="1">
-        <v>2</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
+      <c r="F37" s="22">
+        <v>3</v>
+      </c>
+      <c r="G37" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="38" spans="3:7" x14ac:dyDescent="0.25">
@@ -75680,14 +75689,14 @@
       <c r="D38" s="1">
         <v>0</v>
       </c>
-      <c r="E38" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F38" s="22">
-        <v>3</v>
-      </c>
-      <c r="G38" s="22">
-        <v>0.75</v>
+      <c r="E38" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F38" s="1">
+        <v>1</v>
+      </c>
+      <c r="G38" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="3:7" x14ac:dyDescent="0.25">
@@ -75701,10 +75710,10 @@
         <v>503</v>
       </c>
       <c r="F39" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="40" spans="3:7" x14ac:dyDescent="0.25">
@@ -75714,13 +75723,13 @@
       <c r="D40" s="1">
         <v>0</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F40" s="1">
-        <v>2</v>
-      </c>
-      <c r="G40" s="1">
+      <c r="F40" s="22">
+        <v>3</v>
+      </c>
+      <c r="G40" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75731,14 +75740,14 @@
       <c r="D41" s="1">
         <v>0</v>
       </c>
-      <c r="E41" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F41" s="22">
-        <v>3</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.5</v>
+      <c r="E41" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F41" s="1">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1">
+        <v>2.5</v>
       </c>
     </row>
     <row r="42" spans="3:7" x14ac:dyDescent="0.25">
@@ -75752,10 +75761,10 @@
         <v>1179</v>
       </c>
       <c r="F42" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" s="1">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="43" spans="3:7" x14ac:dyDescent="0.25">
@@ -75765,13 +75774,13 @@
       <c r="D43" s="1">
         <v>0</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F43" s="1">
-        <v>2</v>
-      </c>
-      <c r="G43" s="1">
+      <c r="F43" s="22">
+        <v>3</v>
+      </c>
+      <c r="G43" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75782,14 +75791,14 @@
       <c r="D44" s="1">
         <v>0</v>
       </c>
-      <c r="E44" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F44" s="22">
+      <c r="E44" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F44" s="1">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1">
         <v>3</v>
-      </c>
-      <c r="G44" s="22">
-        <v>1.5</v>
       </c>
     </row>
     <row r="45" spans="3:7" x14ac:dyDescent="0.25">
@@ -75803,10 +75812,10 @@
         <v>505</v>
       </c>
       <c r="F45" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="46" spans="3:7" x14ac:dyDescent="0.25">
@@ -75816,13 +75825,13 @@
       <c r="D46" s="1">
         <v>0</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F46" s="1">
-        <v>2</v>
-      </c>
-      <c r="G46" s="1">
+      <c r="F46" s="22">
+        <v>3</v>
+      </c>
+      <c r="G46" s="22">
         <v>1.5</v>
       </c>
     </row>
@@ -75833,14 +75842,14 @@
       <c r="D47" s="1">
         <v>0</v>
       </c>
-      <c r="E47" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F47" s="22">
-        <v>3</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.5</v>
+      <c r="E47" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F47" s="1">
+        <v>1</v>
+      </c>
+      <c r="G47" s="1">
+        <v>3.5</v>
       </c>
     </row>
     <row r="48" spans="3:7" x14ac:dyDescent="0.25">
@@ -75854,10 +75863,10 @@
         <v>506</v>
       </c>
       <c r="F48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="1">
-        <v>3.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="3:7" x14ac:dyDescent="0.25">
@@ -75867,14 +75876,14 @@
       <c r="D49" s="1">
         <v>0</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F49" s="1">
-        <v>2</v>
-      </c>
-      <c r="G49" s="1">
-        <v>2</v>
+      <c r="F49" s="22">
+        <v>3</v>
+      </c>
+      <c r="G49" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="50" spans="3:7" x14ac:dyDescent="0.25">
@@ -75884,14 +75893,14 @@
       <c r="D50" s="1">
         <v>0</v>
       </c>
-      <c r="E50" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F50" s="22">
-        <v>3</v>
-      </c>
-      <c r="G50" s="22">
-        <v>1.5</v>
+      <c r="E50" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F50" s="1">
+        <v>1</v>
+      </c>
+      <c r="G50" s="1">
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="3:7" x14ac:dyDescent="0.25">
@@ -75905,10 +75914,10 @@
         <v>507</v>
       </c>
       <c r="F51" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="3:7" x14ac:dyDescent="0.25">
@@ -75918,14 +75927,14 @@
       <c r="D52" s="1">
         <v>0</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F52" s="1">
-        <v>2</v>
-      </c>
-      <c r="G52" s="1">
-        <v>2</v>
+      <c r="F52" s="22">
+        <v>3</v>
+      </c>
+      <c r="G52" s="22">
+        <v>1.5</v>
       </c>
     </row>
     <row r="53" spans="3:7" x14ac:dyDescent="0.25">
@@ -75935,14 +75944,14 @@
       <c r="D53" s="1">
         <v>0</v>
       </c>
-      <c r="E53" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F53" s="22">
-        <v>3</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.5</v>
+      <c r="E53" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F53" s="1">
+        <v>1</v>
+      </c>
+      <c r="G53" s="1">
+        <v>5</v>
       </c>
     </row>
     <row r="54" spans="3:7" x14ac:dyDescent="0.25">
@@ -75956,10 +75965,10 @@
         <v>508</v>
       </c>
       <c r="F54" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G54" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="3:7" x14ac:dyDescent="0.25">
@@ -75969,82 +75978,82 @@
       <c r="D55" s="1">
         <v>0</v>
       </c>
-      <c r="E55" s="1" t="s">
+      <c r="E55" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55" s="22">
+        <v>3</v>
+      </c>
+      <c r="G55" s="22">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D56" s="234">
+        <v>0</v>
+      </c>
+      <c r="E56" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F56" s="234">
+        <v>1</v>
+      </c>
+      <c r="G56" s="234">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D57" s="234">
+        <v>0</v>
+      </c>
+      <c r="E57" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F57" s="234">
         <v>2</v>
       </c>
-      <c r="G55" s="1">
+      <c r="G57" s="234">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D56" s="1">
-        <v>0</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F56" s="22">
+      <c r="D58" s="22">
+        <v>0</v>
+      </c>
+      <c r="E58" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="F58" s="22">
         <v>3</v>
       </c>
-      <c r="G56" s="22">
+      <c r="G58" s="22">
         <v>1.5</v>
       </c>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D57" s="1">
-        <v>0</v>
-      </c>
-      <c r="E57" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F57" s="1">
-        <v>1</v>
-      </c>
-      <c r="G57" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="1">
-        <v>0</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F58" s="1">
-        <v>2</v>
-      </c>
-      <c r="G58" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="22">
-        <v>0</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="F59" s="22">
-        <v>3</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.5</v>
+      <c r="E59" s="1" t="s">
+        <v>1178</v>
+      </c>
+      <c r="F59" s="1">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="3:7" x14ac:dyDescent="0.25">
@@ -76058,10 +76067,10 @@
         <v>1178</v>
       </c>
       <c r="F60" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60" s="1">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="61" spans="3:7" x14ac:dyDescent="0.25">
@@ -76071,13 +76080,13 @@
       <c r="D61" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="22" t="s">
         <v>1178</v>
       </c>
-      <c r="F61" s="1">
-        <v>2</v>
-      </c>
-      <c r="G61" s="1">
+      <c r="F61" s="22">
+        <v>3</v>
+      </c>
+      <c r="G61" s="22">
         <v>0.75</v>
       </c>
     </row>
@@ -76088,14 +76097,14 @@
       <c r="D62" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E62" s="22" t="s">
-        <v>1178</v>
-      </c>
-      <c r="F62" s="22">
-        <v>3</v>
-      </c>
-      <c r="G62" s="22">
-        <v>0.75</v>
+      <c r="E62" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="F62" s="1">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="63" spans="3:7" x14ac:dyDescent="0.25">
@@ -76109,10 +76118,10 @@
         <v>502</v>
       </c>
       <c r="F63" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G63" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="3:7" x14ac:dyDescent="0.25">
@@ -76122,14 +76131,14 @@
       <c r="D64" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E64" s="1" t="s">
+      <c r="E64" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F64" s="1">
-        <v>2</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
+      <c r="F64" s="22">
+        <v>3</v>
+      </c>
+      <c r="G64" s="22">
+        <v>0.75</v>
       </c>
     </row>
     <row r="65" spans="3:7" x14ac:dyDescent="0.25">
@@ -76139,14 +76148,14 @@
       <c r="D65" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E65" s="22" t="s">
-        <v>502</v>
-      </c>
-      <c r="F65" s="22">
-        <v>3</v>
-      </c>
-      <c r="G65" s="22">
-        <v>0.75</v>
+      <c r="E65" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="F65" s="1">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="66" spans="3:7" x14ac:dyDescent="0.25">
@@ -76160,7 +76169,7 @@
         <v>503</v>
       </c>
       <c r="F66" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="1">
         <v>1.5</v>
@@ -76173,14 +76182,14 @@
       <c r="D67" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E67" s="1" t="s">
+      <c r="E67" s="22" t="s">
         <v>503</v>
       </c>
-      <c r="F67" s="1">
-        <v>2</v>
-      </c>
-      <c r="G67" s="1">
-        <v>1.5</v>
+      <c r="F67" s="22">
+        <v>3</v>
+      </c>
+      <c r="G67" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="3:7" x14ac:dyDescent="0.25">
@@ -76190,14 +76199,14 @@
       <c r="D68" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E68" s="22" t="s">
-        <v>503</v>
-      </c>
-      <c r="F68" s="22">
-        <v>3</v>
-      </c>
-      <c r="G68" s="22">
-        <v>1</v>
+      <c r="E68" s="1" t="s">
+        <v>1179</v>
+      </c>
+      <c r="F68" s="1">
+        <v>1</v>
+      </c>
+      <c r="G68" s="1">
+        <v>1.5</v>
       </c>
     </row>
     <row r="69" spans="3:7" x14ac:dyDescent="0.25">
@@ -76211,7 +76220,7 @@
         <v>1179</v>
       </c>
       <c r="F69" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G69" s="1">
         <v>1.5</v>
@@ -76224,14 +76233,14 @@
       <c r="D70" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="E70" s="22" t="s">
         <v>1179</v>
       </c>
-      <c r="F70" s="1">
-        <v>2</v>
-      </c>
-      <c r="G70" s="1">
-        <v>1.5</v>
+      <c r="F70" s="22">
+        <v>3</v>
+      </c>
+      <c r="G70" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="3:7" x14ac:dyDescent="0.25">
@@ -76241,14 +76250,14 @@
       <c r="D71" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E71" s="22" t="s">
-        <v>1179</v>
-      </c>
-      <c r="F71" s="22">
-        <v>3</v>
-      </c>
-      <c r="G71" s="22">
-        <v>1</v>
+      <c r="E71" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="F71" s="1">
+        <v>1</v>
+      </c>
+      <c r="G71" s="1">
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="3:7" x14ac:dyDescent="0.25">
@@ -76262,10 +76271,10 @@
         <v>505</v>
       </c>
       <c r="F72" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="73" spans="3:7" x14ac:dyDescent="0.25">
@@ -76275,14 +76284,14 @@
       <c r="D73" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E73" s="1" t="s">
+      <c r="E73" s="22" t="s">
         <v>505</v>
       </c>
-      <c r="F73" s="1">
-        <v>2</v>
-      </c>
-      <c r="G73" s="1">
-        <v>1.5</v>
+      <c r="F73" s="22">
+        <v>3</v>
+      </c>
+      <c r="G73" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="3:7" x14ac:dyDescent="0.25">
@@ -76292,14 +76301,14 @@
       <c r="D74" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E74" s="22" t="s">
-        <v>505</v>
-      </c>
-      <c r="F74" s="22">
+      <c r="E74" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="F74" s="1">
+        <v>1</v>
+      </c>
+      <c r="G74" s="1">
         <v>3</v>
-      </c>
-      <c r="G74" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="75" spans="3:7" x14ac:dyDescent="0.25">
@@ -76313,10 +76322,10 @@
         <v>506</v>
       </c>
       <c r="F75" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="76" spans="3:7" x14ac:dyDescent="0.25">
@@ -76326,14 +76335,14 @@
       <c r="D76" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E76" s="1" t="s">
+      <c r="E76" s="22" t="s">
         <v>506</v>
       </c>
-      <c r="F76" s="1">
-        <v>2</v>
-      </c>
-      <c r="G76" s="1">
-        <v>1.5</v>
+      <c r="F76" s="22">
+        <v>3</v>
+      </c>
+      <c r="G76" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="3:7" x14ac:dyDescent="0.25">
@@ -76343,14 +76352,14 @@
       <c r="D77" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E77" s="22" t="s">
-        <v>506</v>
-      </c>
-      <c r="F77" s="22">
+      <c r="E77" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="F77" s="1">
+        <v>1</v>
+      </c>
+      <c r="G77" s="1">
         <v>3</v>
-      </c>
-      <c r="G77" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="78" spans="3:7" x14ac:dyDescent="0.25">
@@ -76364,10 +76373,10 @@
         <v>507</v>
       </c>
       <c r="F78" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="79" spans="3:7" x14ac:dyDescent="0.25">
@@ -76377,14 +76386,14 @@
       <c r="D79" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E79" s="1" t="s">
+      <c r="E79" s="22" t="s">
         <v>507</v>
       </c>
-      <c r="F79" s="1">
-        <v>2</v>
-      </c>
-      <c r="G79" s="1">
-        <v>1.5</v>
+      <c r="F79" s="22">
+        <v>3</v>
+      </c>
+      <c r="G79" s="22">
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="3:7" x14ac:dyDescent="0.25">
@@ -76394,14 +76403,14 @@
       <c r="D80" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E80" s="22" t="s">
-        <v>507</v>
-      </c>
-      <c r="F80" s="22">
+      <c r="E80" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="F80" s="1">
+        <v>1</v>
+      </c>
+      <c r="G80" s="1">
         <v>3</v>
-      </c>
-      <c r="G80" s="22">
-        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
@@ -76415,10 +76424,10 @@
         <v>508</v>
       </c>
       <c r="F81" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G81" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
@@ -76428,104 +76437,92 @@
       <c r="D82" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E82" s="1" t="s">
+      <c r="E82" s="22" t="s">
         <v>508</v>
       </c>
-      <c r="F82" s="1">
+      <c r="F82" s="22">
+        <v>3</v>
+      </c>
+      <c r="G82" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E83" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F83" s="234">
+        <v>1</v>
+      </c>
+      <c r="G83" s="234">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="D84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="E84" s="234" t="s">
+        <v>353</v>
+      </c>
+      <c r="F84" s="234">
         <v>2</v>
       </c>
-      <c r="G82" s="1">
+      <c r="G84" s="234">
         <v>1.5</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C83" s="1" t="s">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="D83" s="1" t="s">
+      <c r="D85" s="4" t="s">
         <v>353</v>
       </c>
-      <c r="E83" s="22" t="s">
-        <v>508</v>
-      </c>
-      <c r="F83" s="22">
+      <c r="E85" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="F85" s="4">
         <v>3</v>
       </c>
-      <c r="G83" s="22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C84" s="1" t="s">
+      <c r="G85" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D84" s="1" t="s">
+      <c r="D86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E84" s="1" t="s">
+      <c r="E86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="F84" s="1">
-        <v>1</v>
-      </c>
-      <c r="G84" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C85" s="1" t="s">
+      <c r="F86" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F85" s="1">
-        <v>2</v>
-      </c>
-      <c r="G85" s="1">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="D86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="E86" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="F86" s="4">
-        <v>3</v>
-      </c>
-      <c r="G86" s="4">
-        <v>1</v>
+      <c r="G86" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="G87" s="1">
-        <v>6</v>
+      <c r="B87" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B88" t="s">
-        <v>50</v>
+      <c r="A88" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -76537,53 +76534,66 @@
       <c r="A90" t="s">
         <v>0</v>
       </c>
+      <c r="B90" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>0</v>
-      </c>
-      <c r="B91" t="s">
-        <v>1159</v>
-      </c>
+      <c r="B91" s="145" t="s">
+        <v>1160</v>
+      </c>
+      <c r="C91" s="145"/>
+      <c r="D91" s="146"/>
+      <c r="E91" s="146"/>
+      <c r="F91" s="146"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B92" s="145" t="s">
-        <v>1160</v>
-      </c>
-      <c r="C92" s="145"/>
-      <c r="D92" s="146"/>
-      <c r="E92" s="146"/>
-      <c r="F92" s="146"/>
+      <c r="C92" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D92" s="229" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E92" s="147" t="s">
+        <v>1162</v>
+      </c>
+      <c r="F92" s="229" t="s">
+        <v>1166</v>
+      </c>
+      <c r="G92" s="148" t="s">
+        <v>1168</v>
+      </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C93" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D93" s="229" t="s">
-        <v>1161</v>
-      </c>
-      <c r="E93" s="147" t="s">
-        <v>1162</v>
-      </c>
-      <c r="F93" s="229" t="s">
-        <v>1166</v>
-      </c>
-      <c r="G93" s="148" t="s">
-        <v>1168</v>
+      <c r="C93" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D93" s="230" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F93" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G93" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C94" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D94" s="230" t="s">
-        <v>1164</v>
-      </c>
-      <c r="E94" s="1" t="s">
+      <c r="D94" s="232" t="str">
+        <f>D93</f>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F94" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G94" s="1">
         <v>1</v>
@@ -76594,17 +76604,17 @@
         <v>353</v>
       </c>
       <c r="D95" s="232" t="str">
-        <f>D94</f>
+        <f t="shared" ref="D95:D98" si="1">D94</f>
         <v>MPassInteg</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F95" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G95" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -76612,17 +76622,17 @@
         <v>353</v>
       </c>
       <c r="D96" s="232" t="str">
-        <f t="shared" ref="D96:D99" si="1">D95</f>
+        <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E96" s="6" t="s">
-        <v>1163</v>
+      <c r="E96" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F96" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G96" s="1">
-        <v>1.1499999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="3:7" x14ac:dyDescent="0.25">
@@ -76633,67 +76643,67 @@
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E97" s="1" t="s">
+      <c r="E97" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F97" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G97" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C98" s="1" t="s">
+      <c r="C98" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D98" s="232" t="str">
+      <c r="D98" s="233" t="str">
         <f t="shared" si="1"/>
         <v>MPassInteg</v>
       </c>
-      <c r="E98" s="6" t="s">
+      <c r="E98" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F98" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G98" s="1">
-        <v>1</v>
+      <c r="F98" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G98" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="99" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C99" s="22" t="s">
+      <c r="C99" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D99" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E99" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F99" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G99" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D99" s="230" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F99" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G99" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C100" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D100" s="230" t="s">
-        <v>1170</v>
-      </c>
-      <c r="E100" s="1" t="s">
+      <c r="D100" s="232" t="str">
+        <f>D99</f>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E100" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F100" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G100" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.25">
@@ -76701,17 +76711,17 @@
         <v>353</v>
       </c>
       <c r="D101" s="232" t="str">
-        <f>D100</f>
+        <f t="shared" ref="D101:D104" si="2">D100</f>
         <v>SPassPrim-PrimTank</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F101" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G101" s="1">
-        <v>1</v>
+        <v>1.1399999999999999</v>
       </c>
     </row>
     <row r="102" spans="3:7" x14ac:dyDescent="0.25">
@@ -76719,17 +76729,17 @@
         <v>353</v>
       </c>
       <c r="D102" s="232" t="str">
-        <f t="shared" ref="D102:D105" si="2">D101</f>
+        <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E102" s="6" t="s">
-        <v>1163</v>
+      <c r="E102" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F102" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G102" s="1">
-        <v>1.1399999999999999</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103" spans="3:7" x14ac:dyDescent="0.25">
@@ -76740,67 +76750,67 @@
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E103" s="1" t="s">
+      <c r="E103" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F103" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G103" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="104" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C104" s="1" t="s">
+      <c r="C104" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D104" s="232" t="str">
+      <c r="D104" s="233" t="str">
         <f t="shared" si="2"/>
         <v>SPassPrim-PrimTank</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="E104" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F104" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G104" s="1">
-        <v>1</v>
+      <c r="F104" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G104" s="22">
+        <v>1.0900000000000001</v>
       </c>
     </row>
     <row r="105" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C105" s="22" t="s">
+      <c r="C105" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D105" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E105" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F105" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G105" s="22">
-        <v>1.0900000000000001</v>
+      <c r="D105" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F105" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G105" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C106" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D106" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="E106" s="1" t="s">
+      <c r="D106" s="232" t="str">
+        <f>D105</f>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E106" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F106" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G106" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.25">
@@ -76808,17 +76818,17 @@
         <v>353</v>
       </c>
       <c r="D107" s="232" t="str">
-        <f>D106</f>
+        <f t="shared" ref="D107:D110" si="3">D106</f>
         <v>MPassPrim-PrimTank</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F107" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G107" s="1">
-        <v>1</v>
+        <v>1.1499999999999999</v>
       </c>
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.25">
@@ -76826,17 +76836,17 @@
         <v>353</v>
       </c>
       <c r="D108" s="232" t="str">
-        <f t="shared" ref="D108:D111" si="3">D107</f>
+        <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E108" s="6" t="s">
-        <v>1163</v>
+      <c r="E108" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F108" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G108" s="1">
-        <v>1.1499999999999999</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.25">
@@ -76847,67 +76857,67 @@
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E109" s="1" t="s">
+      <c r="E109" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F109" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G109" s="1">
-        <v>0.98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C110" s="1" t="s">
+      <c r="C110" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D110" s="232" t="str">
+      <c r="D110" s="233" t="str">
         <f t="shared" si="3"/>
         <v>MPassPrim-PrimTank</v>
       </c>
-      <c r="E110" s="6" t="s">
+      <c r="E110" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F110" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G110" s="1">
-        <v>1</v>
+      <c r="F110" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G110" s="22">
+        <v>1.1200000000000001</v>
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C111" s="22" t="s">
+      <c r="C111" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D111" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E111" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F111" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G111" s="22">
-        <v>1.1200000000000001</v>
+      <c r="D111" s="230" t="s">
+        <v>1172</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F111" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G111" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C112" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D112" s="230" t="s">
-        <v>1172</v>
-      </c>
-      <c r="E112" s="1" t="s">
+      <c r="D112" s="232" t="str">
+        <f>D111</f>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E112" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F112" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G112" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -76915,17 +76925,17 @@
         <v>353</v>
       </c>
       <c r="D113" s="232" t="str">
-        <f>D112</f>
+        <f t="shared" ref="D113:D116" si="4">D112</f>
         <v>SPassPrim-SResist</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F113" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G113" s="1">
-        <v>1</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -76933,17 +76943,17 @@
         <v>353</v>
       </c>
       <c r="D114" s="232" t="str">
-        <f t="shared" ref="D114:D117" si="4">D113</f>
+        <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E114" s="6" t="s">
-        <v>1163</v>
+      <c r="E114" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F114" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G114" s="1">
-        <v>1.08</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
@@ -76954,67 +76964,67 @@
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E115" s="1" t="s">
+      <c r="E115" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F115" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G115" s="1">
-        <v>0.99</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C116" s="1" t="s">
+      <c r="C116" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D116" s="232" t="str">
+      <c r="D116" s="233" t="str">
         <f t="shared" si="4"/>
         <v>SPassPrim-SResist</v>
       </c>
-      <c r="E116" s="6" t="s">
+      <c r="E116" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F116" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G116" s="1">
-        <v>1</v>
+      <c r="F116" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G116" s="22">
+        <v>1.05</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C117" s="22" t="s">
+      <c r="C117" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D117" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E117" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F117" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G117" s="22">
-        <v>1.05</v>
+      <c r="D117" s="230" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>1163</v>
+      </c>
+      <c r="F117" s="230" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G117" s="1">
+        <v>0.96</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D118" s="230" t="s">
-        <v>1173</v>
-      </c>
-      <c r="E118" s="1" t="s">
+      <c r="D118" s="232" t="str">
+        <f>D117</f>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F118" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G118" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
@@ -77022,17 +77032,17 @@
         <v>353</v>
       </c>
       <c r="D119" s="232" t="str">
-        <f>D118</f>
+        <f t="shared" ref="D119:D122" si="5">D118</f>
         <v>SPassPrim-Parallel</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>1163</v>
       </c>
       <c r="F119" s="230" t="s">
-        <v>1167</v>
+        <v>353</v>
       </c>
       <c r="G119" s="1">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -77040,17 +77050,17 @@
         <v>353</v>
       </c>
       <c r="D120" s="232" t="str">
-        <f t="shared" ref="D120:D123" si="5">D119</f>
+        <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E120" s="6" t="s">
-        <v>1163</v>
+      <c r="E120" s="1" t="s">
+        <v>1169</v>
       </c>
       <c r="F120" s="230" t="s">
-        <v>353</v>
+        <v>1165</v>
       </c>
       <c r="G120" s="1">
-        <v>1.1000000000000001</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
@@ -77061,76 +77071,58 @@
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E121" s="1" t="s">
+      <c r="E121" s="6" t="s">
         <v>1169</v>
       </c>
       <c r="F121" s="230" t="s">
-        <v>1165</v>
+        <v>1167</v>
       </c>
       <c r="G121" s="1">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C122" s="1" t="s">
+      <c r="C122" s="22" t="s">
         <v>353</v>
       </c>
-      <c r="D122" s="232" t="str">
+      <c r="D122" s="233" t="str">
         <f t="shared" si="5"/>
         <v>SPassPrim-Parallel</v>
       </c>
-      <c r="E122" s="6" t="s">
+      <c r="E122" s="113" t="s">
         <v>1169</v>
       </c>
-      <c r="F122" s="230" t="s">
-        <v>1167</v>
-      </c>
-      <c r="G122" s="1">
-        <v>1</v>
+      <c r="F122" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G122" s="22">
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C123" s="22" t="s">
+      <c r="C123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="D123" s="233" t="str">
-        <f t="shared" si="5"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E123" s="113" t="s">
-        <v>1169</v>
-      </c>
-      <c r="F123" s="231" t="s">
+      <c r="D123" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="G123" s="22">
-        <v>1.1000000000000001</v>
+      <c r="E123" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F123" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G123" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E124" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F124" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G124" s="1">
-        <v>1</v>
+      <c r="B124" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B125" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="A125" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>